<commit_message>
Patička: platform by filipmracek.com, proměnné {rok} a {web}
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011AtHpjbqs9iMR23airjHG2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D79"/>
+  <dimension ref="A1:D87"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1279,7 +1279,7 @@
       </c>
       <c r="D46" s="6" t="inlineStr">
         <is>
-          <t>drobné: © 2026 Universal Website</t>
+          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
@@ -1381,74 +1381,105 @@
     <row r="56">
       <c r="A56" s="3" t="inlineStr">
         <is>
-          <t>Obrázky a média</t>
-        </is>
-      </c>
-    </row>
-    <row r="57" ht="28" customHeight="1">
+          <t>Proměnné</t>
+        </is>
+      </c>
+    </row>
+    <row r="57" ht="30" customHeight="1">
       <c r="A57" s="2" t="inlineStr">
         <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B57" s="2" t="inlineStr">
-        <is>
-          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
-        </is>
-      </c>
-    </row>
-    <row r="58" ht="28" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B58" s="2" t="inlineStr">
-        <is>
-          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
-        </is>
-      </c>
-    </row>
-    <row r="59" ht="28" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B59" s="2" t="inlineStr">
-        <is>
-          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="60" ht="28" customHeight="1">
-      <c r="A60" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B60" s="2" t="inlineStr">
-        <is>
-          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
-        </is>
-      </c>
-    </row>
-    <row r="61" ht="28" customHeight="1">
-      <c r="A61" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B61" s="2" t="inlineStr">
-        <is>
-          <t>Videa dávejte na YouTube nebo Vimeo a do stránky vložte odkaz.</t>
+          <t>Do kteréhokoli textu můžete napsat proměnnou ve složených závorkách. Web ji při sestavení nahradí.</t>
+        </is>
+      </c>
+    </row>
+    <row r="58">
+      <c r="A58" s="4" t="inlineStr">
+        <is>
+          <t>proměnná</t>
+        </is>
+      </c>
+      <c r="B58" s="4" t="inlineStr">
+        <is>
+          <t>anglicky</t>
+        </is>
+      </c>
+      <c r="C58" s="4" t="inlineStr">
+        <is>
+          <t>co se dosadí</t>
+        </is>
+      </c>
+      <c r="D58" s="4" t="inlineStr">
+        <is>
+          <t>příklad</t>
+        </is>
+      </c>
+    </row>
+    <row r="59">
+      <c r="A59" s="6" t="inlineStr">
+        <is>
+          <t>{rok}</t>
+        </is>
+      </c>
+      <c r="B59" s="5" t="inlineStr">
+        <is>
+          <t>{year}</t>
+        </is>
+      </c>
+      <c r="C59" s="5" t="inlineStr">
+        <is>
+          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
+        </is>
+      </c>
+      <c r="D59" s="6" t="inlineStr">
+        <is>
+          <t>drobné: © {rok} {web}</t>
+        </is>
+      </c>
+    </row>
+    <row r="60">
+      <c r="A60" s="6" t="inlineStr">
+        <is>
+          <t>{web}</t>
+        </is>
+      </c>
+      <c r="B60" s="5" t="inlineStr">
+        <is>
+          <t>{site}</t>
+        </is>
+      </c>
+      <c r="C60" s="5" t="inlineStr">
+        <is>
+          <t>Název webu z listu site (site_name).</t>
+        </is>
+      </c>
+      <c r="D60" s="6" t="inlineStr">
+        <is>
+          <t>text: Vítejte na {web}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="61">
+      <c r="A61" s="6" t="inlineStr">
+        <is>
+          <t>(c)</t>
+        </is>
+      </c>
+      <c r="B61" s="5" t="inlineStr"/>
+      <c r="C61" s="5" t="inlineStr">
+        <is>
+          <t>Napíše se jako ©.</t>
+        </is>
+      </c>
+      <c r="D61" s="6" t="inlineStr">
+        <is>
+          <t>drobné: (c) {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="3" t="inlineStr">
         <is>
-          <t>Publikování</t>
+          <t>Obrázky a média</t>
         </is>
       </c>
     </row>
@@ -1460,7 +1491,7 @@
       </c>
       <c r="B64" s="2" t="inlineStr">
         <is>
-          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
+          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1472,7 +1503,7 @@
       </c>
       <c r="B65" s="2" t="inlineStr">
         <is>
-          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
         </is>
       </c>
     </row>
@@ -1484,38 +1515,38 @@
       </c>
       <c r="B66" s="2" t="inlineStr">
         <is>
-          <t>Dokud nekliknete na Publikovat, návštěvníci vidí předchozí verzi. Upravovat tedy můžete v klidu.</t>
-        </is>
-      </c>
-    </row>
-    <row r="68">
-      <c r="A68" s="3" t="inlineStr">
-        <is>
-          <t>Pravidla</t>
-        </is>
-      </c>
-    </row>
-    <row r="69" ht="28" customHeight="1">
-      <c r="A69" s="2" t="inlineStr">
+          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="67" ht="28" customHeight="1">
+      <c r="A67" s="2" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B69" s="2" t="inlineStr">
-        <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
-        </is>
-      </c>
-    </row>
-    <row r="70" ht="28" customHeight="1">
-      <c r="A70" s="2" t="inlineStr">
+      <c r="B67" s="2" t="inlineStr">
+        <is>
+          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+        </is>
+      </c>
+    </row>
+    <row r="68" ht="28" customHeight="1">
+      <c r="A68" s="2" t="inlineStr">
         <is>
           <t>•</t>
         </is>
       </c>
-      <c r="B70" s="2" t="inlineStr">
-        <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+      <c r="B68" s="2" t="inlineStr">
+        <is>
+          <t>Videa dávejte na YouTube nebo Vimeo a do stránky vložte odkaz.</t>
+        </is>
+      </c>
+    </row>
+    <row r="70">
+      <c r="A70" s="3" t="inlineStr">
+        <is>
+          <t>Publikování</t>
         </is>
       </c>
     </row>
@@ -1527,7 +1558,7 @@
       </c>
       <c r="B71" s="2" t="inlineStr">
         <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1539,7 +1570,7 @@
       </c>
       <c r="B72" s="2" t="inlineStr">
         <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
         </is>
       </c>
     </row>
@@ -1551,90 +1582,171 @@
       </c>
       <c r="B73" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>Dokud nekliknete na Publikovat, návštěvníci vidí předchozí verzi. Upravovat tedy můžete v klidu.</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="3" t="inlineStr">
         <is>
+          <t>Pravidla</t>
+        </is>
+      </c>
+    </row>
+    <row r="76" ht="28" customHeight="1">
+      <c r="A76" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B76" s="2" t="inlineStr">
+        <is>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
+        </is>
+      </c>
+    </row>
+    <row r="77" ht="28" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B77" s="2" t="inlineStr">
+        <is>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="78" ht="28" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B78" s="2" t="inlineStr">
+        <is>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="79" ht="28" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B79" s="2" t="inlineStr">
+        <is>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="80" ht="28" customHeight="1">
+      <c r="A80" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B80" s="2" t="inlineStr">
+        <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81" ht="28" customHeight="1">
+      <c r="A81" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B81" s="2" t="inlineStr">
+        <is>
+          <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
+        <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="8" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
         </is>
       </c>
-      <c r="B76" s="2" t="inlineStr"/>
-      <c r="C76" s="2" t="inlineStr">
+      <c r="B84" s="2" t="inlineStr"/>
+      <c r="C84" s="2" t="inlineStr">
         <is>
           <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="2" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="2" t="inlineStr">
         <is>
           <t>bílé buňky</t>
         </is>
       </c>
-      <c r="B77" s="2" t="inlineStr"/>
-      <c r="C77" s="2" t="inlineStr">
+      <c r="B85" s="2" t="inlineStr"/>
+      <c r="C85" s="2" t="inlineStr">
         <is>
           <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="9" t="inlineStr">
+    <row r="86">
+      <c r="A86" s="9" t="inlineStr">
         <is>
           <t>šedé buňky</t>
         </is>
       </c>
-      <c r="B78" s="2" t="inlineStr"/>
-      <c r="C78" s="2" t="inlineStr">
+      <c r="B86" s="2" t="inlineStr"/>
+      <c r="C86" s="2" t="inlineStr">
         <is>
           <t>Poznámky pro vás. Na webu se neobjeví.</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="2" t="inlineStr">
+    <row r="87">
+      <c r="A87" s="2" t="inlineStr">
         <is>
           <t>roletky</t>
         </is>
       </c>
-      <c r="B79" s="2" t="inlineStr"/>
-      <c r="C79" s="2" t="inlineStr">
+      <c r="B87" s="2" t="inlineStr"/>
+      <c r="C87" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="19">
-    <mergeCell ref="B60:D60"/>
-    <mergeCell ref="B61:D61"/>
-    <mergeCell ref="B57:D57"/>
+  <mergeCells count="21">
+    <mergeCell ref="B67:D67"/>
     <mergeCell ref="B73:D73"/>
-    <mergeCell ref="B69:D69"/>
+    <mergeCell ref="B78:D78"/>
     <mergeCell ref="A34:D34"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A24:D24"/>
     <mergeCell ref="B65:D65"/>
+    <mergeCell ref="B68:D68"/>
     <mergeCell ref="B64:D64"/>
+    <mergeCell ref="B80:D80"/>
+    <mergeCell ref="B76:D76"/>
+    <mergeCell ref="B79:D79"/>
     <mergeCell ref="A54:D54"/>
     <mergeCell ref="A25:D25"/>
+    <mergeCell ref="B81:D81"/>
     <mergeCell ref="B72:D72"/>
-    <mergeCell ref="B59:D59"/>
     <mergeCell ref="B66:D66"/>
     <mergeCell ref="B71:D71"/>
-    <mergeCell ref="B58:D58"/>
-    <mergeCell ref="B70:D70"/>
+    <mergeCell ref="A57:D57"/>
     <mergeCell ref="A2:D2"/>
+    <mergeCell ref="B77:D77"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -5973,12 +6085,12 @@
       </c>
       <c r="B9" s="5" t="inlineStr">
         <is>
-          <t>drobné: © 2026 Universal Website · Postaveno z tabulky</t>
+          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
       <c r="C9" s="13" t="inlineStr">
         <is>
-          <t>Patička na každé stránce. Stejný zápis jako content.</t>
+          <t>Patička na každé stránce. Stejný zápis jako content. {rok} je vždy aktuální rok, {web} je site_name. Prázdné = © rok a název webu.</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Ukázkový web fyzioterapeutky, styl seznamu faq, oprava poměru stran obrázků v kartách
Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_011AtHpjbqs9iMR23airjHG2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -996,12 +996,12 @@
       <c r="B31" s="5" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr">
         <is>
-          <t>steps / cards / bullets</t>
+          <t>steps / cards / bullets / faq</t>
         </is>
       </c>
       <c r="D31" s="5" t="inlineStr">
         <is>
-          <t>steps čísluje karty podle order; cards bez čísel</t>
+          <t>steps čísluje karty podle order; cards bez čísel; faq = rozbalovací otázky (title = otázka, text = odpověď)</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Kontaktní formulář: formulář: kontakt, příjem v Apps Scriptu
Formulář se odesílá do webové aplikace řídicí tabulky (doPost), ta přečte
adresu form_email z tabulky klienta a pošle zprávu e-mailem s odpovědí na
odesílatele. Ochrana: skryté pole, minimální doba vyplnění, 30 zpráv za
hodinu na web, záznam bez osobních údajů v listu formulare.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_01Q5FKadqaA35T8pcZXYtkma
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D106"/>
+  <dimension ref="A1:D107"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -671,7 +671,7 @@
       </c>
       <c r="D10" s="5" t="inlineStr">
         <is>
-          <t>Widgety, formuláře, cokoli vlastního.</t>
+          <t>Widgety a cokoli vlastního.</t>
         </is>
       </c>
     </row>
@@ -887,483 +887,505 @@
         </is>
       </c>
     </row>
-    <row r="24" ht="30" customHeight="1">
-      <c r="A24" s="2" t="inlineStr">
-        <is>
-          <t>Jedno slovo bez mezer, které odpovídá existujícímu id, se vždy vezme jako odkaz na ten obsah. Cokoli jiného se zobrazí jako text.</t>
+    <row r="23">
+      <c r="A23" s="6" t="inlineStr">
+        <is>
+          <t>formulář:</t>
+        </is>
+      </c>
+      <c r="B23" s="5" t="inlineStr">
+        <is>
+          <t>form:</t>
+        </is>
+      </c>
+      <c r="C23" s="5" t="inlineStr">
+        <is>
+          <t>kontakt (zprávy chodí na form_email z listu site)</t>
+        </is>
+      </c>
+      <c r="D23" s="6" t="inlineStr">
+        <is>
+          <t>formulář: kontakt</t>
         </is>
       </c>
     </row>
     <row r="25" ht="30" customHeight="1">
       <c r="A25" s="2" t="inlineStr">
         <is>
+          <t>Jedno slovo bez mezer, které odpovídá existujícímu id, se vždy vezme jako odkaz na ten obsah. Cokoli jiného se zobrazí jako text.</t>
+        </is>
+      </c>
+    </row>
+    <row r="26" ht="30" customHeight="1">
+      <c r="A26" s="2" t="inlineStr">
+        <is>
           <t>Za svislou čáru | můžete napsat styl. Bez stylu se použije výchozí (první v tabulce níže).</t>
         </is>
       </c>
     </row>
-    <row r="26">
-      <c r="A26" s="4" t="inlineStr">
+    <row r="27">
+      <c r="A27" s="4" t="inlineStr">
         <is>
           <t>obsah</t>
         </is>
       </c>
-      <c r="B26" s="4" t="inlineStr"/>
-      <c r="C26" s="4" t="inlineStr">
+      <c r="B27" s="4" t="inlineStr"/>
+      <c r="C27" s="4" t="inlineStr">
         <is>
           <t>styly</t>
         </is>
       </c>
-      <c r="D26" s="4" t="inlineStr">
+      <c r="D27" s="4" t="inlineStr">
         <is>
           <t>co znamenají</t>
-        </is>
-      </c>
-    </row>
-    <row r="27">
-      <c r="A27" s="5" t="inlineStr">
-        <is>
-          <t>text</t>
-        </is>
-      </c>
-      <c r="B27" s="5" t="inlineStr"/>
-      <c r="C27" s="5" t="inlineStr">
-        <is>
-          <t>normal / wide / centered / large</t>
-        </is>
-      </c>
-      <c r="D27" s="5" t="inlineStr">
-        <is>
-          <t>large = větší písmo pro výrazné sdělení</t>
         </is>
       </c>
     </row>
     <row r="28">
       <c r="A28" s="5" t="inlineStr">
         <is>
-          <t>obrázek</t>
+          <t>text</t>
         </is>
       </c>
       <c r="B28" s="5" t="inlineStr"/>
       <c r="C28" s="5" t="inlineStr">
         <is>
-          <t>inset / full</t>
+          <t>normal / wide / centered / large</t>
         </is>
       </c>
       <c r="D28" s="5" t="inlineStr">
         <is>
-          <t>full = přes celou šířku stránky</t>
+          <t>large = větší písmo pro výrazné sdělení</t>
         </is>
       </c>
     </row>
     <row r="29">
       <c r="A29" s="5" t="inlineStr">
         <is>
-          <t>galerie</t>
+          <t>obrázek</t>
         </is>
       </c>
       <c r="B29" s="5" t="inlineStr"/>
       <c r="C29" s="5" t="inlineStr">
         <is>
-          <t>grid / row</t>
+          <t>inset / full</t>
         </is>
       </c>
       <c r="D29" s="5" t="inlineStr">
         <is>
-          <t>row = řada, která se posouvá do strany</t>
+          <t>full = přes celou šířku stránky</t>
         </is>
       </c>
     </row>
     <row r="30">
       <c r="A30" s="5" t="inlineStr">
         <is>
-          <t>video</t>
+          <t>galerie</t>
         </is>
       </c>
       <c r="B30" s="5" t="inlineStr"/>
       <c r="C30" s="5" t="inlineStr">
         <is>
-          <t>normal / wide</t>
-        </is>
-      </c>
-      <c r="D30" s="5" t="inlineStr"/>
+          <t>grid / row</t>
+        </is>
+      </c>
+      <c r="D30" s="5" t="inlineStr">
+        <is>
+          <t>row = řada, která se posouvá do strany</t>
+        </is>
+      </c>
     </row>
     <row r="31">
       <c r="A31" s="5" t="inlineStr">
         <is>
-          <t>seznam</t>
+          <t>video</t>
         </is>
       </c>
       <c r="B31" s="5" t="inlineStr"/>
       <c r="C31" s="5" t="inlineStr">
         <is>
+          <t>normal / wide</t>
+        </is>
+      </c>
+      <c r="D31" s="5" t="inlineStr"/>
+    </row>
+    <row r="32">
+      <c r="A32" s="5" t="inlineStr">
+        <is>
+          <t>seznam</t>
+        </is>
+      </c>
+      <c r="B32" s="5" t="inlineStr"/>
+      <c r="C32" s="5" t="inlineStr">
+        <is>
           <t>steps / cards / bullets / faq</t>
         </is>
       </c>
-      <c r="D31" s="5" t="inlineStr">
+      <c r="D32" s="5" t="inlineStr">
         <is>
           <t>steps čísluje karty podle order; cards bez čísel; faq = rozbalovací otázky (title = otázka, text = odpověď)</t>
         </is>
       </c>
     </row>
-    <row r="33">
-      <c r="A33" s="3" t="inlineStr">
+    <row r="34">
+      <c r="A34" s="3" t="inlineStr">
         <is>
           <t>Formátování textu</t>
         </is>
       </c>
     </row>
-    <row r="34" ht="30" customHeight="1">
-      <c r="A34" s="2" t="inlineStr">
+    <row r="35" ht="30" customHeight="1">
+      <c r="A35" s="2" t="inlineStr">
         <is>
           <t>Tato slova můžete psát přímo v content stránky i v listu texts. Vše v jedné buňce, každou část na nový řádek.</t>
         </is>
       </c>
     </row>
-    <row r="35">
-      <c r="A35" s="4" t="inlineStr">
+    <row r="36">
+      <c r="A36" s="4" t="inlineStr">
         <is>
           <t>klíčové slovo</t>
         </is>
       </c>
-      <c r="B35" s="4" t="inlineStr">
+      <c r="B36" s="4" t="inlineStr">
         <is>
           <t>anglicky</t>
         </is>
       </c>
-      <c r="C35" s="4" t="inlineStr">
+      <c r="C36" s="4" t="inlineStr">
         <is>
           <t>co vytvoří</t>
         </is>
       </c>
-      <c r="D35" s="4" t="inlineStr">
+      <c r="D36" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="36">
-      <c r="A36" s="6" t="inlineStr">
-        <is>
-          <t>úvod:</t>
-        </is>
-      </c>
-      <c r="B36" s="5" t="inlineStr">
-        <is>
-          <t>lead:</t>
-        </is>
-      </c>
-      <c r="C36" s="5" t="inlineStr">
-        <is>
-          <t>Velký úvodní odstavec</t>
-        </is>
-      </c>
-      <c r="D36" s="6" t="inlineStr">
-        <is>
-          <t>úvod: Každá stránka se čte jako běžný web.</t>
         </is>
       </c>
     </row>
     <row r="37">
       <c r="A37" s="6" t="inlineStr">
         <is>
-          <t>text:</t>
+          <t>úvod:</t>
         </is>
       </c>
       <c r="B37" s="5" t="inlineStr">
         <is>
-          <t>text:</t>
+          <t>lead:</t>
         </is>
       </c>
       <c r="C37" s="5" t="inlineStr">
         <is>
-          <t>Odstavec. Prázdný řádek uvnitř = nový odstavec.</t>
+          <t>Velký úvodní odstavec</t>
         </is>
       </c>
       <c r="D37" s="6" t="inlineStr">
         <is>
-          <t>text: Ostatní stránky nejsou vidět.</t>
+          <t>úvod: Každá stránka se čte jako běžný web.</t>
         </is>
       </c>
     </row>
     <row r="38">
       <c r="A38" s="6" t="inlineStr">
         <is>
-          <t>nadpis:</t>
+          <t>text:</t>
         </is>
       </c>
       <c r="B38" s="5" t="inlineStr">
         <is>
-          <t>heading:</t>
+          <t>text:</t>
         </is>
       </c>
       <c r="C38" s="5" t="inlineStr">
         <is>
-          <t>Nadpis oddílu</t>
+          <t>Odstavec. Prázdný řádek uvnitř = nový odstavec.</t>
         </is>
       </c>
       <c r="D38" s="6" t="inlineStr">
         <is>
-          <t>nadpis: Proč je to rychlé</t>
+          <t>text: Ostatní stránky nejsou vidět.</t>
         </is>
       </c>
     </row>
     <row r="39">
       <c r="A39" s="6" t="inlineStr">
         <is>
-          <t>mezititulek:</t>
+          <t>nadpis:</t>
         </is>
       </c>
       <c r="B39" s="5" t="inlineStr">
         <is>
-          <t>subheading:</t>
+          <t>heading:</t>
         </is>
       </c>
       <c r="C39" s="5" t="inlineStr">
         <is>
-          <t>Menší nadpis</t>
+          <t>Nadpis oddílu</t>
         </is>
       </c>
       <c r="D39" s="6" t="inlineStr">
         <is>
-          <t>mezititulek: Zkuste ho přerušit</t>
+          <t>nadpis: Proč je to rychlé</t>
         </is>
       </c>
     </row>
     <row r="40">
       <c r="A40" s="6" t="inlineStr">
         <is>
-          <t>citace:</t>
+          <t>mezititulek:</t>
         </is>
       </c>
       <c r="B40" s="5" t="inlineStr">
         <is>
-          <t>quote:</t>
+          <t>subheading:</t>
         </is>
       </c>
       <c r="C40" s="5" t="inlineStr">
         <is>
-          <t>Zvýrazněná citace</t>
+          <t>Menší nadpis</t>
         </is>
       </c>
       <c r="D40" s="6" t="inlineStr">
         <is>
-          <t>citace: Ať to působí jako skutečná stránka.</t>
+          <t>mezititulek: Zkuste ho přerušit</t>
         </is>
       </c>
     </row>
     <row r="41">
       <c r="A41" s="6" t="inlineStr">
         <is>
-          <t>autor:</t>
+          <t>citace:</t>
         </is>
       </c>
       <c r="B41" s="5" t="inlineStr">
         <is>
-          <t>author:</t>
+          <t>quote:</t>
         </is>
       </c>
       <c r="C41" s="5" t="inlineStr">
         <is>
-          <t>Kdo to řekl; patří k citaci nad ním</t>
+          <t>Zvýrazněná citace</t>
         </is>
       </c>
       <c r="D41" s="6" t="inlineStr">
         <is>
-          <t>autor: Studio</t>
+          <t>citace: Ať to působí jako skutečná stránka.</t>
         </is>
       </c>
     </row>
     <row r="42">
       <c r="A42" s="6" t="inlineStr">
         <is>
-          <t>seznam:</t>
+          <t>autor:</t>
         </is>
       </c>
       <c r="B42" s="5" t="inlineStr">
         <is>
-          <t>list:</t>
+          <t>author:</t>
         </is>
       </c>
       <c r="C42" s="5" t="inlineStr">
         <is>
-          <t>Odrážky oddělené ; nebo řádky začínající -</t>
+          <t>Kdo to řekl; patří k citaci nad ním</t>
         </is>
       </c>
       <c r="D42" s="6" t="inlineStr">
         <is>
-          <t>seznam: rychlé; lehké; z tabulky</t>
+          <t>autor: Studio</t>
         </is>
       </c>
     </row>
     <row r="43">
       <c r="A43" s="6" t="inlineStr">
         <is>
-          <t>poznámka:</t>
+          <t>seznam:</t>
         </is>
       </c>
       <c r="B43" s="5" t="inlineStr">
         <is>
-          <t>note:</t>
+          <t>list:</t>
         </is>
       </c>
       <c r="C43" s="5" t="inlineStr">
         <is>
-          <t>Rámeček s poznámkou</t>
+          <t>Odrážky oddělené ; nebo řádky začínající -</t>
         </is>
       </c>
       <c r="D43" s="6" t="inlineStr">
         <is>
-          <t>poznámka: Tabulka se čte při sestavení.</t>
+          <t>seznam: rychlé; lehké; z tabulky</t>
         </is>
       </c>
     </row>
     <row r="44">
       <c r="A44" s="6" t="inlineStr">
         <is>
-          <t>tlačítko:</t>
+          <t>poznámka:</t>
         </is>
       </c>
       <c r="B44" s="5" t="inlineStr">
         <is>
-          <t>button:</t>
+          <t>note:</t>
         </is>
       </c>
       <c r="C44" s="5" t="inlineStr">
         <is>
-          <t>Tlačítko: popis -&gt; odkaz</t>
+          <t>Rámeček s poznámkou</t>
         </is>
       </c>
       <c r="D44" s="6" t="inlineStr">
         <is>
-          <t>tlačítko: Napište nám -&gt; https://example.com</t>
+          <t>poznámka: Tabulka se čte při sestavení.</t>
         </is>
       </c>
     </row>
     <row r="45">
       <c r="A45" s="6" t="inlineStr">
         <is>
-          <t>oddělovač:</t>
+          <t>tlačítko:</t>
         </is>
       </c>
       <c r="B45" s="5" t="inlineStr">
         <is>
-          <t>divider:</t>
+          <t>button:</t>
         </is>
       </c>
       <c r="C45" s="5" t="inlineStr">
         <is>
-          <t>Tenká čára; za dvojtečkou nic</t>
+          <t>Tlačítko: popis -&gt; odkaz</t>
         </is>
       </c>
       <c r="D45" s="6" t="inlineStr">
         <is>
-          <t>oddělovač:</t>
+          <t>tlačítko: Napište nám -&gt; https://example.com</t>
         </is>
       </c>
     </row>
     <row r="46">
       <c r="A46" s="6" t="inlineStr">
         <is>
+          <t>oddělovač:</t>
+        </is>
+      </c>
+      <c r="B46" s="5" t="inlineStr">
+        <is>
+          <t>divider:</t>
+        </is>
+      </c>
+      <c r="C46" s="5" t="inlineStr">
+        <is>
+          <t>Tenká čára; za dvojtečkou nic</t>
+        </is>
+      </c>
+      <c r="D46" s="6" t="inlineStr">
+        <is>
+          <t>oddělovač:</t>
+        </is>
+      </c>
+    </row>
+    <row r="47">
+      <c r="A47" s="6" t="inlineStr">
+        <is>
           <t>drobné:</t>
         </is>
       </c>
-      <c r="B46" s="5" t="inlineStr">
+      <c r="B47" s="5" t="inlineStr">
         <is>
           <t>small:</t>
         </is>
       </c>
-      <c r="C46" s="5" t="inlineStr">
+      <c r="C47" s="5" t="inlineStr">
         <is>
           <t>Drobný text</t>
         </is>
       </c>
-      <c r="D46" s="6" t="inlineStr">
+      <c r="D47" s="6" t="inlineStr">
         <is>
           <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
-    <row r="48">
-      <c r="A48" s="4" t="inlineStr">
+    <row r="49">
+      <c r="A49" s="4" t="inlineStr">
         <is>
           <t>uvnitř textu</t>
         </is>
       </c>
-      <c r="B48" s="4" t="inlineStr"/>
-      <c r="C48" s="4" t="inlineStr">
+      <c r="B49" s="4" t="inlineStr"/>
+      <c r="C49" s="4" t="inlineStr">
         <is>
           <t>výsledek</t>
         </is>
       </c>
-      <c r="D48" s="4" t="inlineStr">
+      <c r="D49" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="49">
-      <c r="A49" s="6" t="inlineStr">
-        <is>
-          <t>**slova**</t>
-        </is>
-      </c>
-      <c r="B49" s="5" t="inlineStr"/>
-      <c r="C49" s="5" t="inlineStr">
-        <is>
-          <t>tučně</t>
-        </is>
-      </c>
-      <c r="D49" s="6" t="inlineStr">
-        <is>
-          <t>stoh **změní směr**</t>
         </is>
       </c>
     </row>
     <row r="50">
       <c r="A50" s="6" t="inlineStr">
         <is>
-          <t>*slova*</t>
+          <t>**slova**</t>
         </is>
       </c>
       <c r="B50" s="5" t="inlineStr"/>
       <c r="C50" s="5" t="inlineStr">
         <is>
-          <t>kurzíva</t>
+          <t>tučně</t>
         </is>
       </c>
       <c r="D50" s="6" t="inlineStr">
         <is>
-          <t>z *Google Sheets*</t>
+          <t>stoh **změní směr**</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>[slova](odkaz)</t>
+          <t>*slova*</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
       <c r="C51" s="5" t="inlineStr">
         <is>
+          <t>kurzíva</t>
+        </is>
+      </c>
+      <c r="D51" s="6" t="inlineStr">
+        <is>
+          <t>z *Google Sheets*</t>
+        </is>
+      </c>
+    </row>
+    <row r="52">
+      <c r="A52" s="6" t="inlineStr">
+        <is>
+          <t>[slova](odkaz)</t>
+        </is>
+      </c>
+      <c r="B52" s="5" t="inlineStr"/>
+      <c r="C52" s="5" t="inlineStr">
+        <is>
           <t>odkaz</t>
         </is>
       </c>
-      <c r="D51" s="6" t="inlineStr">
+      <c r="D52" s="6" t="inlineStr">
         <is>
           <t>viz [naše studio](https://example.com)</t>
         </is>
       </c>
     </row>
-    <row r="53">
-      <c r="A53" s="3" t="inlineStr">
+    <row r="54">
+      <c r="A54" s="3" t="inlineStr">
         <is>
           <t>Celá stránka v jedné buňce</t>
         </is>
       </c>
     </row>
-    <row r="54" ht="150" customHeight="1">
-      <c r="A54" s="7" t="inlineStr">
+    <row r="55" ht="150" customHeight="1">
+      <c r="A55" s="7" t="inlineStr">
         <is>
           <t>úvod: Až bude pohyb sedět, přijde platforma pod ním.
 text: t-intro
@@ -1378,422 +1400,410 @@
         </is>
       </c>
     </row>
-    <row r="56">
-      <c r="A56" s="3" t="inlineStr">
+    <row r="57">
+      <c r="A57" s="3" t="inlineStr">
         <is>
           <t>Barevné profily (styles › color_profile)</t>
         </is>
       </c>
     </row>
-    <row r="57" ht="42" customHeight="1">
-      <c r="A57" s="2" t="inlineStr">
+    <row r="58" ht="42" customHeight="1">
+      <c r="A58" s="2" t="inlineStr">
         <is>
           <t>V listu styles vyberte v řádku color_profile jeden profil. Pozadí zůstává živé a jemně proměnlivé, profil mu dává základní tón. Kromě manual profily nepoužívají sloupec hue ani barvy textu z listu styles.</t>
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="4" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="4" t="inlineStr">
         <is>
           <t>profil</t>
         </is>
       </c>
-      <c r="B58" s="4" t="inlineStr"/>
-      <c r="C58" s="4" t="inlineStr">
+      <c r="B59" s="4" t="inlineStr"/>
+      <c r="C59" s="4" t="inlineStr">
         <is>
           <t>jak působí</t>
         </is>
       </c>
-      <c r="D58" s="4" t="inlineStr">
+      <c r="D59" s="4" t="inlineStr">
         <is>
           <t>barvy</t>
-        </is>
-      </c>
-    </row>
-    <row r="59">
-      <c r="A59" s="5" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="B59" s="5" t="inlineStr"/>
-      <c r="C59" s="5" t="inlineStr">
-        <is>
-          <t>Barvu každé stránky určuje sloupec hue v listu pages.</t>
-        </is>
-      </c>
-      <c r="D59" s="5" t="inlineStr">
-        <is>
-          <t>podle vás</t>
         </is>
       </c>
     </row>
     <row r="60">
       <c r="A60" s="5" t="inlineStr">
         <is>
-          <t>terakota</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="B60" s="5" t="inlineStr"/>
       <c r="C60" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
+          <t>Barvu každé stránky určuje sloupec hue v listu pages.</t>
         </is>
       </c>
       <c r="D60" s="5" t="inlineStr">
         <is>
-          <t>#C8643B</t>
+          <t>podle vás</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>jantar</t>
+          <t>terakota</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr"/>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>#D9932E</t>
+          <t>#C8643B</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>koral</t>
+          <t>jantar</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr"/>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>#E8715A</t>
+          <t>#D9932E</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>broskev</t>
+          <t>koral</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr"/>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>#E89B7A</t>
+          <t>#E8715A</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>karamel</t>
+          <t>broskev</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr"/>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>#B9773F</t>
+          <t>#E89B7A</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>ruze</t>
+          <t>karamel</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>#C97B84</t>
+          <t>#B9773F</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>vinova</t>
+          <t>ruze</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr"/>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>#9E3B5A</t>
+          <t>#C97B84</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>pisek</t>
+          <t>vinova</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr"/>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>#C9A77A</t>
+          <t>#9E3B5A</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>seda</t>
+          <t>pisek</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr"/>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>#9C9C9E</t>
+          <t>#C9A77A</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>tron</t>
+          <t>seda</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr"/>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
+          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>#00E5FF · #FF7A1A</t>
+          <t>#9C9C9E</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>soumrak</t>
+          <t>tron</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr"/>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy se střídají po stránkách. Tlumená korálová, indigo, tyrkys, zlatá.</t>
+          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>#D98B6A #7C78C8 #5BA8A0 #D9B86C</t>
+          <t>#00E5FF · #FF7A1A</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>zeme</t>
+          <t>soumrak</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr"/>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy. Mech, okr, cihla, jezerní modrá.</t>
+          <t>Čtyři barvy se střídají po stránkách. Tlumená korálová, indigo, tyrkys, zlatá.</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>#8FBF6F #E9A23B #C9583E #4F86C6</t>
+          <t>#D98B6A #7C78C8 #5BA8A0 #D9B86C</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>pastel</t>
+          <t>zeme</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr"/>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy. Tlumená růžová, aqua, levandulová, světlá citronová.</t>
+          <t>Čtyři barvy. Mech, okr, cihla, jezerní modrá.</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>#D9A3B8 #9CCBCF #A3B4D9 #DCD9A8</t>
+          <t>#8FBF6F #E9A23B #C9583E #4F86C6</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>sever</t>
+          <t>pastel</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr"/>
       <c r="C73" s="5" t="inlineStr">
         <is>
+          <t>Čtyři barvy. Tlumená růžová, aqua, levandulová, světlá citronová.</t>
+        </is>
+      </c>
+      <c r="D73" s="5" t="inlineStr">
+        <is>
+          <t>#D9A3B8 #9CCBCF #A3B4D9 #DCD9A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="74">
+      <c r="A74" s="5" t="inlineStr">
+        <is>
+          <t>sever</t>
+        </is>
+      </c>
+      <c r="B74" s="5" t="inlineStr"/>
+      <c r="C74" s="5" t="inlineStr">
+        <is>
           <t>Čtyři barvy. Severská modrá, šalvěj, pšeničná, tlumená červená.</t>
         </is>
       </c>
-      <c r="D73" s="5" t="inlineStr">
+      <c r="D74" s="5" t="inlineStr">
         <is>
           <t>#88C0D0 #A3BE8C #EBCB8B #BF616A</t>
         </is>
       </c>
     </row>
-    <row r="75">
-      <c r="A75" s="3" t="inlineStr">
+    <row r="76">
+      <c r="A76" s="3" t="inlineStr">
         <is>
           <t>Proměnné</t>
         </is>
       </c>
     </row>
-    <row r="76" ht="30" customHeight="1">
-      <c r="A76" s="2" t="inlineStr">
+    <row r="77" ht="30" customHeight="1">
+      <c r="A77" s="2" t="inlineStr">
         <is>
           <t>Do kteréhokoli textu můžete napsat proměnnou ve složených závorkách. Web ji při sestavení nahradí.</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="4" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="4" t="inlineStr">
         <is>
           <t>proměnná</t>
         </is>
       </c>
-      <c r="B77" s="4" t="inlineStr">
+      <c r="B78" s="4" t="inlineStr">
         <is>
           <t>anglicky</t>
         </is>
       </c>
-      <c r="C77" s="4" t="inlineStr">
+      <c r="C78" s="4" t="inlineStr">
         <is>
           <t>co se dosadí</t>
         </is>
       </c>
-      <c r="D77" s="4" t="inlineStr">
+      <c r="D78" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="78">
-      <c r="A78" s="6" t="inlineStr">
-        <is>
-          <t>{rok}</t>
-        </is>
-      </c>
-      <c r="B78" s="5" t="inlineStr">
-        <is>
-          <t>{year}</t>
-        </is>
-      </c>
-      <c r="C78" s="5" t="inlineStr">
-        <is>
-          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
-        </is>
-      </c>
-      <c r="D78" s="6" t="inlineStr">
-        <is>
-          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="79">
       <c r="A79" s="6" t="inlineStr">
         <is>
-          <t>{web}</t>
+          <t>{rok}</t>
         </is>
       </c>
       <c r="B79" s="5" t="inlineStr">
         <is>
-          <t>{site}</t>
+          <t>{year}</t>
         </is>
       </c>
       <c r="C79" s="5" t="inlineStr">
         <is>
-          <t>Název webu z listu site (site_name).</t>
+          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
         </is>
       </c>
       <c r="D79" s="6" t="inlineStr">
         <is>
-          <t>text: Vítejte na {web}.</t>
+          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
+          <t>{web}</t>
+        </is>
+      </c>
+      <c r="B80" s="5" t="inlineStr">
+        <is>
+          <t>{site}</t>
+        </is>
+      </c>
+      <c r="C80" s="5" t="inlineStr">
+        <is>
+          <t>Název webu z listu site (site_name).</t>
+        </is>
+      </c>
+      <c r="D80" s="6" t="inlineStr">
+        <is>
+          <t>text: Vítejte na {web}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="81">
+      <c r="A81" s="6" t="inlineStr">
+        <is>
           <t>(c)</t>
         </is>
       </c>
-      <c r="B80" s="5" t="inlineStr"/>
-      <c r="C80" s="5" t="inlineStr">
+      <c r="B81" s="5" t="inlineStr"/>
+      <c r="C81" s="5" t="inlineStr">
         <is>
           <t>Napíše se jako ©.</t>
         </is>
       </c>
-      <c r="D80" s="6" t="inlineStr">
+      <c r="D81" s="6" t="inlineStr">
         <is>
           <t>drobné: (c) {rok} {web}</t>
         </is>
       </c>
     </row>
-    <row r="82">
-      <c r="A82" s="3" t="inlineStr">
+    <row r="83">
+      <c r="A83" s="3" t="inlineStr">
         <is>
           <t>Obrázky a média</t>
-        </is>
-      </c>
-    </row>
-    <row r="83" ht="28" customHeight="1">
-      <c r="A83" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B83" s="2" t="inlineStr">
-        <is>
-          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1805,7 +1815,7 @@
       </c>
       <c r="B84" s="2" t="inlineStr">
         <is>
-          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
+          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1817,7 +1827,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
+          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
         </is>
       </c>
     </row>
@@ -1829,7 +1839,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
         </is>
       </c>
     </row>
@@ -1841,26 +1851,26 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
+          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+        </is>
+      </c>
+    </row>
+    <row r="88" ht="28" customHeight="1">
+      <c r="A88" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B88" s="2" t="inlineStr">
+        <is>
           <t>Videa dávejte na YouTube nebo Vimeo a do stránky vložte odkaz.</t>
         </is>
       </c>
     </row>
-    <row r="89">
-      <c r="A89" s="3" t="inlineStr">
+    <row r="90">
+      <c r="A90" s="3" t="inlineStr">
         <is>
           <t>Publikování</t>
-        </is>
-      </c>
-    </row>
-    <row r="90" ht="28" customHeight="1">
-      <c r="A90" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B90" s="2" t="inlineStr">
-        <is>
-          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1872,7 +1882,7 @@
       </c>
       <c r="B91" s="2" t="inlineStr">
         <is>
-          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1884,26 +1894,26 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
+          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+        </is>
+      </c>
+    </row>
+    <row r="93" ht="28" customHeight="1">
+      <c r="A93" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B93" s="2" t="inlineStr">
+        <is>
           <t>Dokud nekliknete na Publikovat, návštěvníci vidí předchozí verzi. Upravovat tedy můžete v klidu.</t>
         </is>
       </c>
     </row>
-    <row r="94">
-      <c r="A94" s="3" t="inlineStr">
+    <row r="95">
+      <c r="A95" s="3" t="inlineStr">
         <is>
           <t>Pravidla</t>
-        </is>
-      </c>
-    </row>
-    <row r="95" ht="28" customHeight="1">
-      <c r="A95" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B95" s="2" t="inlineStr">
-        <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -1915,7 +1925,7 @@
       </c>
       <c r="B96" s="2" t="inlineStr">
         <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -1927,7 +1937,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
         </is>
       </c>
     </row>
@@ -1939,7 +1949,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
         </is>
       </c>
     </row>
@@ -1951,7 +1961,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
         </is>
       </c>
     </row>
@@ -1963,64 +1973,76 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
           <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
         </is>
       </c>
     </row>
-    <row r="102">
-      <c r="A102" s="3" t="inlineStr">
+    <row r="103">
+      <c r="A103" s="3" t="inlineStr">
         <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="8" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
-        </is>
-      </c>
-      <c r="B103" s="2" t="inlineStr"/>
-      <c r="C103" s="2" t="inlineStr">
-        <is>
-          <t>Obsah stránky a texty. Tady skládáte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>bílé buňky</t>
         </is>
       </c>
       <c r="B104" s="2" t="inlineStr"/>
       <c r="C104" s="2" t="inlineStr">
         <is>
-          <t>Nastavení a údaje.</t>
+          <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
     <row r="105">
-      <c r="A105" s="9" t="inlineStr">
-        <is>
-          <t>šedé buňky</t>
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>bílé buňky</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr"/>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Poznámky pro vás. Na webu se neobjeví.</t>
+          <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>roletky</t>
+      <c r="A106" s="9" t="inlineStr">
+        <is>
+          <t>šedé buňky</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
+        <is>
+          <t>Poznámky pro vás. Na webu se neobjeví.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>roletky</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr"/>
+      <c r="C107" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
@@ -2029,26 +2051,26 @@
   </sheetData>
   <mergeCells count="22">
     <mergeCell ref="B98:D98"/>
+    <mergeCell ref="A35:D35"/>
+    <mergeCell ref="B101:D101"/>
+    <mergeCell ref="B88:D88"/>
     <mergeCell ref="B87:D87"/>
-    <mergeCell ref="A34:D34"/>
+    <mergeCell ref="A58:D58"/>
+    <mergeCell ref="A77:D77"/>
     <mergeCell ref="B99:D99"/>
     <mergeCell ref="B84:D84"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="B92:D92"/>
-    <mergeCell ref="A24:D24"/>
-    <mergeCell ref="B83:D83"/>
-    <mergeCell ref="B95:D95"/>
     <mergeCell ref="B85:D85"/>
-    <mergeCell ref="A54:D54"/>
     <mergeCell ref="B97:D97"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="B100:D100"/>
     <mergeCell ref="B91:D91"/>
-    <mergeCell ref="B90:D90"/>
+    <mergeCell ref="A26:D26"/>
+    <mergeCell ref="B93:D93"/>
+    <mergeCell ref="A55:D55"/>
     <mergeCell ref="B96:D96"/>
-    <mergeCell ref="A57:D57"/>
     <mergeCell ref="A2:D2"/>
-    <mergeCell ref="A76:D76"/>
     <mergeCell ref="B86:D86"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
@@ -6398,7 +6420,17 @@
       </c>
     </row>
     <row r="10">
-      <c r="C10" s="15" t="n"/>
+      <c r="A10" s="11" t="inlineStr">
+        <is>
+          <t>form_email</t>
+        </is>
+      </c>
+      <c r="B10" s="5" t="inlineStr"/>
+      <c r="C10" s="13" t="inlineStr">
+        <is>
+          <t>Kam chodí zprávy z formuláře (formulář: kontakt). Na webu se nezobrazí. Více adres oddělte čárkou.</t>
+        </is>
+      </c>
     </row>
     <row r="11">
       <c r="C11" s="15" t="n"/>

</xml_diff>

<commit_message>
Víc místa nad nadpisy, nový blok mezera:
Nadpisy dosud neměly horní okraj vůbec (přebíjelo ho .inner > *).
mezera: / space: vloží volné místo, prázdné = běžné, velká / malá.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fseswgzcM5xGxappQkPY2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D107"/>
+  <dimension ref="A1:D108"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1286,106 +1286,128 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
+          <t>mezera:</t>
+        </is>
+      </c>
+      <c r="B47" s="5" t="inlineStr">
+        <is>
+          <t>space:</t>
+        </is>
+      </c>
+      <c r="C47" s="5" t="inlineStr">
+        <is>
+          <t>Volné místo. Prázdné = běžná, nebo velká / malá</t>
+        </is>
+      </c>
+      <c r="D47" s="6" t="inlineStr">
+        <is>
+          <t>mezera: velká</t>
+        </is>
+      </c>
+    </row>
+    <row r="48">
+      <c r="A48" s="6" t="inlineStr">
+        <is>
           <t>drobné:</t>
         </is>
       </c>
-      <c r="B47" s="5" t="inlineStr">
+      <c r="B48" s="5" t="inlineStr">
         <is>
           <t>small:</t>
         </is>
       </c>
-      <c r="C47" s="5" t="inlineStr">
+      <c r="C48" s="5" t="inlineStr">
         <is>
           <t>Drobný text</t>
         </is>
       </c>
-      <c r="D47" s="6" t="inlineStr">
+      <c r="D48" s="6" t="inlineStr">
         <is>
           <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
-    <row r="49">
-      <c r="A49" s="4" t="inlineStr">
+    <row r="50">
+      <c r="A50" s="4" t="inlineStr">
         <is>
           <t>uvnitř textu</t>
         </is>
       </c>
-      <c r="B49" s="4" t="inlineStr"/>
-      <c r="C49" s="4" t="inlineStr">
+      <c r="B50" s="4" t="inlineStr"/>
+      <c r="C50" s="4" t="inlineStr">
         <is>
           <t>výsledek</t>
         </is>
       </c>
-      <c r="D49" s="4" t="inlineStr">
+      <c r="D50" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="50">
-      <c r="A50" s="6" t="inlineStr">
-        <is>
-          <t>**slova**</t>
-        </is>
-      </c>
-      <c r="B50" s="5" t="inlineStr"/>
-      <c r="C50" s="5" t="inlineStr">
-        <is>
-          <t>tučně</t>
-        </is>
-      </c>
-      <c r="D50" s="6" t="inlineStr">
-        <is>
-          <t>stoh **změní směr**</t>
         </is>
       </c>
     </row>
     <row r="51">
       <c r="A51" s="6" t="inlineStr">
         <is>
-          <t>*slova*</t>
+          <t>**slova**</t>
         </is>
       </c>
       <c r="B51" s="5" t="inlineStr"/>
       <c r="C51" s="5" t="inlineStr">
         <is>
-          <t>kurzíva</t>
+          <t>tučně</t>
         </is>
       </c>
       <c r="D51" s="6" t="inlineStr">
         <is>
-          <t>z *Google Sheets*</t>
+          <t>stoh **změní směr**</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>[slova](odkaz)</t>
+          <t>*slova*</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr">
         <is>
+          <t>kurzíva</t>
+        </is>
+      </c>
+      <c r="D52" s="6" t="inlineStr">
+        <is>
+          <t>z *Google Sheets*</t>
+        </is>
+      </c>
+    </row>
+    <row r="53">
+      <c r="A53" s="6" t="inlineStr">
+        <is>
+          <t>[slova](odkaz)</t>
+        </is>
+      </c>
+      <c r="B53" s="5" t="inlineStr"/>
+      <c r="C53" s="5" t="inlineStr">
+        <is>
           <t>odkaz</t>
         </is>
       </c>
-      <c r="D52" s="6" t="inlineStr">
+      <c r="D53" s="6" t="inlineStr">
         <is>
           <t>viz [naše studio](https://example.com)</t>
         </is>
       </c>
     </row>
-    <row r="54">
-      <c r="A54" s="3" t="inlineStr">
+    <row r="55">
+      <c r="A55" s="3" t="inlineStr">
         <is>
           <t>Celá stránka v jedné buňce</t>
         </is>
       </c>
     </row>
-    <row r="55" ht="150" customHeight="1">
-      <c r="A55" s="7" t="inlineStr">
+    <row r="56" ht="150" customHeight="1">
+      <c r="A56" s="7" t="inlineStr">
         <is>
           <t>úvod: Až bude pohyb sedět, přijde platforma pod ním.
 text: t-intro
@@ -1400,422 +1422,410 @@
         </is>
       </c>
     </row>
-    <row r="57">
-      <c r="A57" s="3" t="inlineStr">
+    <row r="58">
+      <c r="A58" s="3" t="inlineStr">
         <is>
           <t>Barevné profily (styles › color_profile)</t>
         </is>
       </c>
     </row>
-    <row r="58" ht="42" customHeight="1">
-      <c r="A58" s="2" t="inlineStr">
+    <row r="59" ht="42" customHeight="1">
+      <c r="A59" s="2" t="inlineStr">
         <is>
           <t>V listu styles vyberte v řádku color_profile jeden profil. Pozadí zůstává živé a jemně proměnlivé, profil mu dává základní tón. Kromě manual profily nepoužívají sloupec hue ani barvy textu z listu styles.</t>
         </is>
       </c>
     </row>
-    <row r="59">
-      <c r="A59" s="4" t="inlineStr">
+    <row r="60">
+      <c r="A60" s="4" t="inlineStr">
         <is>
           <t>profil</t>
         </is>
       </c>
-      <c r="B59" s="4" t="inlineStr"/>
-      <c r="C59" s="4" t="inlineStr">
+      <c r="B60" s="4" t="inlineStr"/>
+      <c r="C60" s="4" t="inlineStr">
         <is>
           <t>jak působí</t>
         </is>
       </c>
-      <c r="D59" s="4" t="inlineStr">
+      <c r="D60" s="4" t="inlineStr">
         <is>
           <t>barvy</t>
-        </is>
-      </c>
-    </row>
-    <row r="60">
-      <c r="A60" s="5" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="B60" s="5" t="inlineStr"/>
-      <c r="C60" s="5" t="inlineStr">
-        <is>
-          <t>Barvu každé stránky určuje sloupec hue v listu pages.</t>
-        </is>
-      </c>
-      <c r="D60" s="5" t="inlineStr">
-        <is>
-          <t>podle vás</t>
         </is>
       </c>
     </row>
     <row r="61">
       <c r="A61" s="5" t="inlineStr">
         <is>
-          <t>terakota</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="B61" s="5" t="inlineStr"/>
       <c r="C61" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
+          <t>Barvu každé stránky určuje sloupec hue v listu pages.</t>
         </is>
       </c>
       <c r="D61" s="5" t="inlineStr">
         <is>
-          <t>#C8643B</t>
+          <t>podle vás</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>jantar</t>
+          <t>terakota</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr"/>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>#D9932E</t>
+          <t>#C8643B</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>koral</t>
+          <t>jantar</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr"/>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>#E8715A</t>
+          <t>#D9932E</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>broskev</t>
+          <t>koral</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr"/>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>#E89B7A</t>
+          <t>#E8715A</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>karamel</t>
+          <t>broskev</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>#B9773F</t>
+          <t>#E89B7A</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>ruze</t>
+          <t>karamel</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr"/>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>#C97B84</t>
+          <t>#B9773F</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>vinova</t>
+          <t>ruze</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr"/>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>#9E3B5A</t>
+          <t>#C97B84</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>pisek</t>
+          <t>vinova</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr"/>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>#C9A77A</t>
+          <t>#9E3B5A</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>seda</t>
+          <t>pisek</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr"/>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>#9C9C9E</t>
+          <t>#C9A77A</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>tron</t>
+          <t>seda</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr"/>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
+          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>#00E5FF · #FF7A1A</t>
+          <t>#9C9C9E</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>soumrak</t>
+          <t>tron</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr"/>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy se střídají po stránkách. Tlumená korálová, indigo, tyrkys, zlatá.</t>
+          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>#D98B6A #7C78C8 #5BA8A0 #D9B86C</t>
+          <t>#00E5FF · #FF7A1A</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>zeme</t>
+          <t>soumrak</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr"/>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy. Mech, okr, cihla, jezerní modrá.</t>
+          <t>Čtyři barvy se střídají po stránkách. Tlumená korálová, indigo, tyrkys, zlatá.</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>#8FBF6F #E9A23B #C9583E #4F86C6</t>
+          <t>#D98B6A #7C78C8 #5BA8A0 #D9B86C</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>pastel</t>
+          <t>zeme</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr"/>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy. Tlumená růžová, aqua, levandulová, světlá citronová.</t>
+          <t>Čtyři barvy. Mech, okr, cihla, jezerní modrá.</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>#D9A3B8 #9CCBCF #A3B4D9 #DCD9A8</t>
+          <t>#8FBF6F #E9A23B #C9583E #4F86C6</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>sever</t>
+          <t>pastel</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr"/>
       <c r="C74" s="5" t="inlineStr">
         <is>
+          <t>Čtyři barvy. Tlumená růžová, aqua, levandulová, světlá citronová.</t>
+        </is>
+      </c>
+      <c r="D74" s="5" t="inlineStr">
+        <is>
+          <t>#D9A3B8 #9CCBCF #A3B4D9 #DCD9A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="75">
+      <c r="A75" s="5" t="inlineStr">
+        <is>
+          <t>sever</t>
+        </is>
+      </c>
+      <c r="B75" s="5" t="inlineStr"/>
+      <c r="C75" s="5" t="inlineStr">
+        <is>
           <t>Čtyři barvy. Severská modrá, šalvěj, pšeničná, tlumená červená.</t>
         </is>
       </c>
-      <c r="D74" s="5" t="inlineStr">
+      <c r="D75" s="5" t="inlineStr">
         <is>
           <t>#88C0D0 #A3BE8C #EBCB8B #BF616A</t>
         </is>
       </c>
     </row>
-    <row r="76">
-      <c r="A76" s="3" t="inlineStr">
+    <row r="77">
+      <c r="A77" s="3" t="inlineStr">
         <is>
           <t>Proměnné</t>
         </is>
       </c>
     </row>
-    <row r="77" ht="30" customHeight="1">
-      <c r="A77" s="2" t="inlineStr">
+    <row r="78" ht="30" customHeight="1">
+      <c r="A78" s="2" t="inlineStr">
         <is>
           <t>Do kteréhokoli textu můžete napsat proměnnou ve složených závorkách. Web ji při sestavení nahradí.</t>
         </is>
       </c>
     </row>
-    <row r="78">
-      <c r="A78" s="4" t="inlineStr">
+    <row r="79">
+      <c r="A79" s="4" t="inlineStr">
         <is>
           <t>proměnná</t>
         </is>
       </c>
-      <c r="B78" s="4" t="inlineStr">
+      <c r="B79" s="4" t="inlineStr">
         <is>
           <t>anglicky</t>
         </is>
       </c>
-      <c r="C78" s="4" t="inlineStr">
+      <c r="C79" s="4" t="inlineStr">
         <is>
           <t>co se dosadí</t>
         </is>
       </c>
-      <c r="D78" s="4" t="inlineStr">
+      <c r="D79" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="79">
-      <c r="A79" s="6" t="inlineStr">
-        <is>
-          <t>{rok}</t>
-        </is>
-      </c>
-      <c r="B79" s="5" t="inlineStr">
-        <is>
-          <t>{year}</t>
-        </is>
-      </c>
-      <c r="C79" s="5" t="inlineStr">
-        <is>
-          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
-        </is>
-      </c>
-      <c r="D79" s="6" t="inlineStr">
-        <is>
-          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="80">
       <c r="A80" s="6" t="inlineStr">
         <is>
-          <t>{web}</t>
+          <t>{rok}</t>
         </is>
       </c>
       <c r="B80" s="5" t="inlineStr">
         <is>
-          <t>{site}</t>
+          <t>{year}</t>
         </is>
       </c>
       <c r="C80" s="5" t="inlineStr">
         <is>
-          <t>Název webu z listu site (site_name).</t>
+          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
         </is>
       </c>
       <c r="D80" s="6" t="inlineStr">
         <is>
-          <t>text: Vítejte na {web}.</t>
+          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
+          <t>{web}</t>
+        </is>
+      </c>
+      <c r="B81" s="5" t="inlineStr">
+        <is>
+          <t>{site}</t>
+        </is>
+      </c>
+      <c r="C81" s="5" t="inlineStr">
+        <is>
+          <t>Název webu z listu site (site_name).</t>
+        </is>
+      </c>
+      <c r="D81" s="6" t="inlineStr">
+        <is>
+          <t>text: Vítejte na {web}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="82">
+      <c r="A82" s="6" t="inlineStr">
+        <is>
           <t>(c)</t>
         </is>
       </c>
-      <c r="B81" s="5" t="inlineStr"/>
-      <c r="C81" s="5" t="inlineStr">
+      <c r="B82" s="5" t="inlineStr"/>
+      <c r="C82" s="5" t="inlineStr">
         <is>
           <t>Napíše se jako ©.</t>
         </is>
       </c>
-      <c r="D81" s="6" t="inlineStr">
+      <c r="D82" s="6" t="inlineStr">
         <is>
           <t>drobné: (c) {rok} {web}</t>
         </is>
       </c>
     </row>
-    <row r="83">
-      <c r="A83" s="3" t="inlineStr">
+    <row r="84">
+      <c r="A84" s="3" t="inlineStr">
         <is>
           <t>Obrázky a média</t>
-        </is>
-      </c>
-    </row>
-    <row r="84" ht="28" customHeight="1">
-      <c r="A84" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B84" s="2" t="inlineStr">
-        <is>
-          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1827,7 +1837,7 @@
       </c>
       <c r="B85" s="2" t="inlineStr">
         <is>
-          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
+          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1839,7 +1849,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
+          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
         </is>
       </c>
     </row>
@@ -1851,7 +1861,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
         </is>
       </c>
     </row>
@@ -1863,26 +1873,26 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
+          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+        </is>
+      </c>
+    </row>
+    <row r="89" ht="28" customHeight="1">
+      <c r="A89" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B89" s="2" t="inlineStr">
+        <is>
           <t>Videa dávejte na YouTube nebo Vimeo a do stránky vložte odkaz.</t>
         </is>
       </c>
     </row>
-    <row r="90">
-      <c r="A90" s="3" t="inlineStr">
+    <row r="91">
+      <c r="A91" s="3" t="inlineStr">
         <is>
           <t>Publikování</t>
-        </is>
-      </c>
-    </row>
-    <row r="91" ht="28" customHeight="1">
-      <c r="A91" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B91" s="2" t="inlineStr">
-        <is>
-          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1894,7 +1904,7 @@
       </c>
       <c r="B92" s="2" t="inlineStr">
         <is>
-          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1906,26 +1916,26 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
+          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+        </is>
+      </c>
+    </row>
+    <row r="94" ht="28" customHeight="1">
+      <c r="A94" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B94" s="2" t="inlineStr">
+        <is>
           <t>Dokud nekliknete na Publikovat, návštěvníci vidí předchozí verzi. Upravovat tedy můžete v klidu.</t>
         </is>
       </c>
     </row>
-    <row r="95">
-      <c r="A95" s="3" t="inlineStr">
+    <row r="96">
+      <c r="A96" s="3" t="inlineStr">
         <is>
           <t>Pravidla</t>
-        </is>
-      </c>
-    </row>
-    <row r="96" ht="28" customHeight="1">
-      <c r="A96" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B96" s="2" t="inlineStr">
-        <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -1937,7 +1947,7 @@
       </c>
       <c r="B97" s="2" t="inlineStr">
         <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -1949,7 +1959,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
         </is>
       </c>
     </row>
@@ -1961,7 +1971,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
         </is>
       </c>
     </row>
@@ -1973,7 +1983,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
         </is>
       </c>
     </row>
@@ -1985,64 +1995,76 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="102" ht="28" customHeight="1">
+      <c r="A102" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B102" s="2" t="inlineStr">
+        <is>
           <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
         </is>
       </c>
     </row>
-    <row r="103">
-      <c r="A103" s="3" t="inlineStr">
+    <row r="104">
+      <c r="A104" s="3" t="inlineStr">
         <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="8" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr"/>
-      <c r="C104" s="2" t="inlineStr">
-        <is>
-          <t>Obsah stránky a texty. Tady skládáte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>bílé buňky</t>
         </is>
       </c>
       <c r="B105" s="2" t="inlineStr"/>
       <c r="C105" s="2" t="inlineStr">
         <is>
-          <t>Nastavení a údaje.</t>
+          <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
     <row r="106">
-      <c r="A106" s="9" t="inlineStr">
-        <is>
-          <t>šedé buňky</t>
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>bílé buňky</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Poznámky pro vás. Na webu se neobjeví.</t>
+          <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="2" t="inlineStr">
-        <is>
-          <t>roletky</t>
+      <c r="A107" s="9" t="inlineStr">
+        <is>
+          <t>šedé buňky</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr"/>
       <c r="C107" s="2" t="inlineStr">
+        <is>
+          <t>Poznámky pro vás. Na webu se neobjeví.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>roletky</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr"/>
+      <c r="C108" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
@@ -2055,21 +2077,21 @@
     <mergeCell ref="B101:D101"/>
     <mergeCell ref="B88:D88"/>
     <mergeCell ref="B87:D87"/>
-    <mergeCell ref="A58:D58"/>
-    <mergeCell ref="A77:D77"/>
     <mergeCell ref="B99:D99"/>
-    <mergeCell ref="B84:D84"/>
     <mergeCell ref="A15:D15"/>
+    <mergeCell ref="A59:D59"/>
     <mergeCell ref="B92:D92"/>
+    <mergeCell ref="B89:D89"/>
+    <mergeCell ref="B94:D94"/>
     <mergeCell ref="B85:D85"/>
+    <mergeCell ref="A78:D78"/>
     <mergeCell ref="B97:D97"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="B100:D100"/>
-    <mergeCell ref="B91:D91"/>
+    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="B102:D102"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="B93:D93"/>
-    <mergeCell ref="A55:D55"/>
-    <mergeCell ref="B96:D96"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B86:D86"/>
   </mergeCells>

</xml_diff>

<commit_message>
Nový blok mapa: (Google Mapy podle adresy v listu site)
mapa: bez hodnoty bere site › address, mapa: <adresa> ukáže jiné místo.
Tmavá verze ladí s webem, | light ji vypne. Mapa se načte, až když je
její stránka vepředu. Pod mapou adresa a odkazy na Mapy a navigaci.
Nová nastavení v site: address, map_zoom.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fseswgzcM5xGxappQkPY2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D108"/>
+  <dimension ref="A1:D109"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1286,128 +1286,150 @@
     <row r="47">
       <c r="A47" s="6" t="inlineStr">
         <is>
-          <t>mezera:</t>
+          <t>mapa:</t>
         </is>
       </c>
       <c r="B47" s="5" t="inlineStr">
         <is>
-          <t>space:</t>
+          <t>map:</t>
         </is>
       </c>
       <c r="C47" s="5" t="inlineStr">
         <is>
-          <t>Volné místo. Prázdné = běžná, nebo velká / malá</t>
+          <t>Mapa Google. Prázdné = adresa z listu site, nebo jiná adresa; | light = světlá</t>
         </is>
       </c>
       <c r="D47" s="6" t="inlineStr">
         <is>
-          <t>mezera: velká</t>
+          <t>mapa:</t>
         </is>
       </c>
     </row>
     <row r="48">
       <c r="A48" s="6" t="inlineStr">
         <is>
+          <t>mezera:</t>
+        </is>
+      </c>
+      <c r="B48" s="5" t="inlineStr">
+        <is>
+          <t>space:</t>
+        </is>
+      </c>
+      <c r="C48" s="5" t="inlineStr">
+        <is>
+          <t>Volné místo. Prázdné = běžná, nebo velká / malá</t>
+        </is>
+      </c>
+      <c r="D48" s="6" t="inlineStr">
+        <is>
+          <t>mezera: velká</t>
+        </is>
+      </c>
+    </row>
+    <row r="49">
+      <c r="A49" s="6" t="inlineStr">
+        <is>
           <t>drobné:</t>
         </is>
       </c>
-      <c r="B48" s="5" t="inlineStr">
+      <c r="B49" s="5" t="inlineStr">
         <is>
           <t>small:</t>
         </is>
       </c>
-      <c r="C48" s="5" t="inlineStr">
+      <c r="C49" s="5" t="inlineStr">
         <is>
           <t>Drobný text</t>
         </is>
       </c>
-      <c r="D48" s="6" t="inlineStr">
+      <c r="D49" s="6" t="inlineStr">
         <is>
           <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
-    <row r="50">
-      <c r="A50" s="4" t="inlineStr">
+    <row r="51">
+      <c r="A51" s="4" t="inlineStr">
         <is>
           <t>uvnitř textu</t>
         </is>
       </c>
-      <c r="B50" s="4" t="inlineStr"/>
-      <c r="C50" s="4" t="inlineStr">
+      <c r="B51" s="4" t="inlineStr"/>
+      <c r="C51" s="4" t="inlineStr">
         <is>
           <t>výsledek</t>
         </is>
       </c>
-      <c r="D50" s="4" t="inlineStr">
+      <c r="D51" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="51">
-      <c r="A51" s="6" t="inlineStr">
-        <is>
-          <t>**slova**</t>
-        </is>
-      </c>
-      <c r="B51" s="5" t="inlineStr"/>
-      <c r="C51" s="5" t="inlineStr">
-        <is>
-          <t>tučně</t>
-        </is>
-      </c>
-      <c r="D51" s="6" t="inlineStr">
-        <is>
-          <t>stoh **změní směr**</t>
         </is>
       </c>
     </row>
     <row r="52">
       <c r="A52" s="6" t="inlineStr">
         <is>
-          <t>*slova*</t>
+          <t>**slova**</t>
         </is>
       </c>
       <c r="B52" s="5" t="inlineStr"/>
       <c r="C52" s="5" t="inlineStr">
         <is>
-          <t>kurzíva</t>
+          <t>tučně</t>
         </is>
       </c>
       <c r="D52" s="6" t="inlineStr">
         <is>
-          <t>z *Google Sheets*</t>
+          <t>stoh **změní směr**</t>
         </is>
       </c>
     </row>
     <row r="53">
       <c r="A53" s="6" t="inlineStr">
         <is>
-          <t>[slova](odkaz)</t>
+          <t>*slova*</t>
         </is>
       </c>
       <c r="B53" s="5" t="inlineStr"/>
       <c r="C53" s="5" t="inlineStr">
         <is>
+          <t>kurzíva</t>
+        </is>
+      </c>
+      <c r="D53" s="6" t="inlineStr">
+        <is>
+          <t>z *Google Sheets*</t>
+        </is>
+      </c>
+    </row>
+    <row r="54">
+      <c r="A54" s="6" t="inlineStr">
+        <is>
+          <t>[slova](odkaz)</t>
+        </is>
+      </c>
+      <c r="B54" s="5" t="inlineStr"/>
+      <c r="C54" s="5" t="inlineStr">
+        <is>
           <t>odkaz</t>
         </is>
       </c>
-      <c r="D53" s="6" t="inlineStr">
+      <c r="D54" s="6" t="inlineStr">
         <is>
           <t>viz [naše studio](https://example.com)</t>
         </is>
       </c>
     </row>
-    <row r="55">
-      <c r="A55" s="3" t="inlineStr">
+    <row r="56">
+      <c r="A56" s="3" t="inlineStr">
         <is>
           <t>Celá stránka v jedné buňce</t>
         </is>
       </c>
     </row>
-    <row r="56" ht="150" customHeight="1">
-      <c r="A56" s="7" t="inlineStr">
+    <row r="57" ht="150" customHeight="1">
+      <c r="A57" s="7" t="inlineStr">
         <is>
           <t>úvod: Až bude pohyb sedět, přijde platforma pod ním.
 text: t-intro
@@ -1422,422 +1444,410 @@
         </is>
       </c>
     </row>
-    <row r="58">
-      <c r="A58" s="3" t="inlineStr">
+    <row r="59">
+      <c r="A59" s="3" t="inlineStr">
         <is>
           <t>Barevné profily (styles › color_profile)</t>
         </is>
       </c>
     </row>
-    <row r="59" ht="42" customHeight="1">
-      <c r="A59" s="2" t="inlineStr">
+    <row r="60" ht="42" customHeight="1">
+      <c r="A60" s="2" t="inlineStr">
         <is>
           <t>V listu styles vyberte v řádku color_profile jeden profil. Pozadí zůstává živé a jemně proměnlivé, profil mu dává základní tón. Kromě manual profily nepoužívají sloupec hue ani barvy textu z listu styles.</t>
         </is>
       </c>
     </row>
-    <row r="60">
-      <c r="A60" s="4" t="inlineStr">
+    <row r="61">
+      <c r="A61" s="4" t="inlineStr">
         <is>
           <t>profil</t>
         </is>
       </c>
-      <c r="B60" s="4" t="inlineStr"/>
-      <c r="C60" s="4" t="inlineStr">
+      <c r="B61" s="4" t="inlineStr"/>
+      <c r="C61" s="4" t="inlineStr">
         <is>
           <t>jak působí</t>
         </is>
       </c>
-      <c r="D60" s="4" t="inlineStr">
+      <c r="D61" s="4" t="inlineStr">
         <is>
           <t>barvy</t>
-        </is>
-      </c>
-    </row>
-    <row r="61">
-      <c r="A61" s="5" t="inlineStr">
-        <is>
-          <t>manual</t>
-        </is>
-      </c>
-      <c r="B61" s="5" t="inlineStr"/>
-      <c r="C61" s="5" t="inlineStr">
-        <is>
-          <t>Barvu každé stránky určuje sloupec hue v listu pages.</t>
-        </is>
-      </c>
-      <c r="D61" s="5" t="inlineStr">
-        <is>
-          <t>podle vás</t>
         </is>
       </c>
     </row>
     <row r="62">
       <c r="A62" s="5" t="inlineStr">
         <is>
-          <t>terakota</t>
+          <t>manual</t>
         </is>
       </c>
       <c r="B62" s="5" t="inlineStr"/>
       <c r="C62" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
+          <t>Barvu každé stránky určuje sloupec hue v listu pages.</t>
         </is>
       </c>
       <c r="D62" s="5" t="inlineStr">
         <is>
-          <t>#C8643B</t>
+          <t>podle vás</t>
         </is>
       </c>
     </row>
     <row r="63">
       <c r="A63" s="5" t="inlineStr">
         <is>
-          <t>jantar</t>
+          <t>terakota</t>
         </is>
       </c>
       <c r="B63" s="5" t="inlineStr"/>
       <c r="C63" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Teplá cihlová.</t>
         </is>
       </c>
       <c r="D63" s="5" t="inlineStr">
         <is>
-          <t>#D9932E</t>
+          <t>#C8643B</t>
         </is>
       </c>
     </row>
     <row r="64">
       <c r="A64" s="5" t="inlineStr">
         <is>
-          <t>koral</t>
+          <t>jantar</t>
         </is>
       </c>
       <c r="B64" s="5" t="inlineStr"/>
       <c r="C64" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Medová, zlatavá.</t>
         </is>
       </c>
       <c r="D64" s="5" t="inlineStr">
         <is>
-          <t>#E8715A</t>
+          <t>#D9932E</t>
         </is>
       </c>
     </row>
     <row r="65">
       <c r="A65" s="5" t="inlineStr">
         <is>
-          <t>broskev</t>
+          <t>koral</t>
         </is>
       </c>
       <c r="B65" s="5" t="inlineStr"/>
       <c r="C65" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Svěží korálová.</t>
         </is>
       </c>
       <c r="D65" s="5" t="inlineStr">
         <is>
-          <t>#E89B7A</t>
+          <t>#E8715A</t>
         </is>
       </c>
     </row>
     <row r="66">
       <c r="A66" s="5" t="inlineStr">
         <is>
-          <t>karamel</t>
+          <t>broskev</t>
         </is>
       </c>
       <c r="B66" s="5" t="inlineStr"/>
       <c r="C66" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Jemná broskvová.</t>
         </is>
       </c>
       <c r="D66" s="5" t="inlineStr">
         <is>
-          <t>#B9773F</t>
+          <t>#E89B7A</t>
         </is>
       </c>
     </row>
     <row r="67">
       <c r="A67" s="5" t="inlineStr">
         <is>
-          <t>ruze</t>
+          <t>karamel</t>
         </is>
       </c>
       <c r="B67" s="5" t="inlineStr"/>
       <c r="C67" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Karamelově hnědá.</t>
         </is>
       </c>
       <c r="D67" s="5" t="inlineStr">
         <is>
-          <t>#C97B84</t>
+          <t>#B9773F</t>
         </is>
       </c>
     </row>
     <row r="68">
       <c r="A68" s="5" t="inlineStr">
         <is>
-          <t>vinova</t>
+          <t>ruze</t>
         </is>
       </c>
       <c r="B68" s="5" t="inlineStr"/>
       <c r="C68" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Prášková růže.</t>
         </is>
       </c>
       <c r="D68" s="5" t="inlineStr">
         <is>
-          <t>#9E3B5A</t>
+          <t>#C97B84</t>
         </is>
       </c>
     </row>
     <row r="69">
       <c r="A69" s="5" t="inlineStr">
         <is>
-          <t>pisek</t>
+          <t>vinova</t>
         </is>
       </c>
       <c r="B69" s="5" t="inlineStr"/>
       <c r="C69" s="5" t="inlineStr">
         <is>
-          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Hluboká vínová.</t>
         </is>
       </c>
       <c r="D69" s="5" t="inlineStr">
         <is>
-          <t>#C9A77A</t>
+          <t>#9E3B5A</t>
         </is>
       </c>
     </row>
     <row r="70">
       <c r="A70" s="5" t="inlineStr">
         <is>
-          <t>seda</t>
+          <t>pisek</t>
         </is>
       </c>
       <c r="B70" s="5" t="inlineStr"/>
       <c r="C70" s="5" t="inlineStr">
         <is>
-          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
+          <t>Jedna barva v odstínech, pozadí v doplňkové barvě. Světlý písek.</t>
         </is>
       </c>
       <c r="D70" s="5" t="inlineStr">
         <is>
-          <t>#9C9C9E</t>
+          <t>#C9A77A</t>
         </is>
       </c>
     </row>
     <row r="71">
       <c r="A71" s="5" t="inlineStr">
         <is>
-          <t>tron</t>
+          <t>seda</t>
         </is>
       </c>
       <c r="B71" s="5" t="inlineStr"/>
       <c r="C71" s="5" t="inlineStr">
         <is>
-          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
+          <t>Stupně šedi, bez barvy. Pozadí v tmavě šedých tónech.</t>
         </is>
       </c>
       <c r="D71" s="5" t="inlineStr">
         <is>
-          <t>#00E5FF · #FF7A1A</t>
+          <t>#9C9C9E</t>
         </is>
       </c>
     </row>
     <row r="72">
       <c r="A72" s="5" t="inlineStr">
         <is>
-          <t>soumrak</t>
+          <t>tron</t>
         </is>
       </c>
       <c r="B72" s="5" t="inlineStr"/>
       <c r="C72" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy se střídají po stránkách. Tlumená korálová, indigo, tyrkys, zlatá.</t>
+          <t>Neonově azurová s oranžovou, záře na hranách, pozadí v modrých a oranžových tónech.</t>
         </is>
       </c>
       <c r="D72" s="5" t="inlineStr">
         <is>
-          <t>#D98B6A #7C78C8 #5BA8A0 #D9B86C</t>
+          <t>#00E5FF · #FF7A1A</t>
         </is>
       </c>
     </row>
     <row r="73">
       <c r="A73" s="5" t="inlineStr">
         <is>
-          <t>zeme</t>
+          <t>soumrak</t>
         </is>
       </c>
       <c r="B73" s="5" t="inlineStr"/>
       <c r="C73" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy. Mech, okr, cihla, jezerní modrá.</t>
+          <t>Čtyři barvy se střídají po stránkách. Tlumená korálová, indigo, tyrkys, zlatá.</t>
         </is>
       </c>
       <c r="D73" s="5" t="inlineStr">
         <is>
-          <t>#8FBF6F #E9A23B #C9583E #4F86C6</t>
+          <t>#D98B6A #7C78C8 #5BA8A0 #D9B86C</t>
         </is>
       </c>
     </row>
     <row r="74">
       <c r="A74" s="5" t="inlineStr">
         <is>
-          <t>pastel</t>
+          <t>zeme</t>
         </is>
       </c>
       <c r="B74" s="5" t="inlineStr"/>
       <c r="C74" s="5" t="inlineStr">
         <is>
-          <t>Čtyři barvy. Tlumená růžová, aqua, levandulová, světlá citronová.</t>
+          <t>Čtyři barvy. Mech, okr, cihla, jezerní modrá.</t>
         </is>
       </c>
       <c r="D74" s="5" t="inlineStr">
         <is>
-          <t>#D9A3B8 #9CCBCF #A3B4D9 #DCD9A8</t>
+          <t>#8FBF6F #E9A23B #C9583E #4F86C6</t>
         </is>
       </c>
     </row>
     <row r="75">
       <c r="A75" s="5" t="inlineStr">
         <is>
-          <t>sever</t>
+          <t>pastel</t>
         </is>
       </c>
       <c r="B75" s="5" t="inlineStr"/>
       <c r="C75" s="5" t="inlineStr">
         <is>
+          <t>Čtyři barvy. Tlumená růžová, aqua, levandulová, světlá citronová.</t>
+        </is>
+      </c>
+      <c r="D75" s="5" t="inlineStr">
+        <is>
+          <t>#D9A3B8 #9CCBCF #A3B4D9 #DCD9A8</t>
+        </is>
+      </c>
+    </row>
+    <row r="76">
+      <c r="A76" s="5" t="inlineStr">
+        <is>
+          <t>sever</t>
+        </is>
+      </c>
+      <c r="B76" s="5" t="inlineStr"/>
+      <c r="C76" s="5" t="inlineStr">
+        <is>
           <t>Čtyři barvy. Severská modrá, šalvěj, pšeničná, tlumená červená.</t>
         </is>
       </c>
-      <c r="D75" s="5" t="inlineStr">
+      <c r="D76" s="5" t="inlineStr">
         <is>
           <t>#88C0D0 #A3BE8C #EBCB8B #BF616A</t>
         </is>
       </c>
     </row>
-    <row r="77">
-      <c r="A77" s="3" t="inlineStr">
+    <row r="78">
+      <c r="A78" s="3" t="inlineStr">
         <is>
           <t>Proměnné</t>
         </is>
       </c>
     </row>
-    <row r="78" ht="30" customHeight="1">
-      <c r="A78" s="2" t="inlineStr">
+    <row r="79" ht="30" customHeight="1">
+      <c r="A79" s="2" t="inlineStr">
         <is>
           <t>Do kteréhokoli textu můžete napsat proměnnou ve složených závorkách. Web ji při sestavení nahradí.</t>
         </is>
       </c>
     </row>
-    <row r="79">
-      <c r="A79" s="4" t="inlineStr">
+    <row r="80">
+      <c r="A80" s="4" t="inlineStr">
         <is>
           <t>proměnná</t>
         </is>
       </c>
-      <c r="B79" s="4" t="inlineStr">
+      <c r="B80" s="4" t="inlineStr">
         <is>
           <t>anglicky</t>
         </is>
       </c>
-      <c r="C79" s="4" t="inlineStr">
+      <c r="C80" s="4" t="inlineStr">
         <is>
           <t>co se dosadí</t>
         </is>
       </c>
-      <c r="D79" s="4" t="inlineStr">
+      <c r="D80" s="4" t="inlineStr">
         <is>
           <t>příklad</t>
-        </is>
-      </c>
-    </row>
-    <row r="80">
-      <c r="A80" s="6" t="inlineStr">
-        <is>
-          <t>{rok}</t>
-        </is>
-      </c>
-      <c r="B80" s="5" t="inlineStr">
-        <is>
-          <t>{year}</t>
-        </is>
-      </c>
-      <c r="C80" s="5" t="inlineStr">
-        <is>
-          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
-        </is>
-      </c>
-      <c r="D80" s="6" t="inlineStr">
-        <is>
-          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="81">
       <c r="A81" s="6" t="inlineStr">
         <is>
-          <t>{web}</t>
+          <t>{rok}</t>
         </is>
       </c>
       <c r="B81" s="5" t="inlineStr">
         <is>
-          <t>{site}</t>
+          <t>{year}</t>
         </is>
       </c>
       <c r="C81" s="5" t="inlineStr">
         <is>
-          <t>Název webu z listu site (site_name).</t>
+          <t>Aktuální rok. Mění se sám, i když web dlouho nepublikujete.</t>
         </is>
       </c>
       <c r="D81" s="6" t="inlineStr">
         <is>
-          <t>text: Vítejte na {web}.</t>
+          <t>drobné: © {rok} {web}</t>
         </is>
       </c>
     </row>
     <row r="82">
       <c r="A82" s="6" t="inlineStr">
         <is>
+          <t>{web}</t>
+        </is>
+      </c>
+      <c r="B82" s="5" t="inlineStr">
+        <is>
+          <t>{site}</t>
+        </is>
+      </c>
+      <c r="C82" s="5" t="inlineStr">
+        <is>
+          <t>Název webu z listu site (site_name).</t>
+        </is>
+      </c>
+      <c r="D82" s="6" t="inlineStr">
+        <is>
+          <t>text: Vítejte na {web}.</t>
+        </is>
+      </c>
+    </row>
+    <row r="83">
+      <c r="A83" s="6" t="inlineStr">
+        <is>
           <t>(c)</t>
         </is>
       </c>
-      <c r="B82" s="5" t="inlineStr"/>
-      <c r="C82" s="5" t="inlineStr">
+      <c r="B83" s="5" t="inlineStr"/>
+      <c r="C83" s="5" t="inlineStr">
         <is>
           <t>Napíše se jako ©.</t>
         </is>
       </c>
-      <c r="D82" s="6" t="inlineStr">
+      <c r="D83" s="6" t="inlineStr">
         <is>
           <t>drobné: (c) {rok} {web}</t>
         </is>
       </c>
     </row>
-    <row r="84">
-      <c r="A84" s="3" t="inlineStr">
+    <row r="85">
+      <c r="A85" s="3" t="inlineStr">
         <is>
           <t>Obrázky a média</t>
-        </is>
-      </c>
-    </row>
-    <row r="85" ht="28" customHeight="1">
-      <c r="A85" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B85" s="2" t="inlineStr">
-        <is>
-          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1849,7 +1859,7 @@
       </c>
       <c r="B86" s="2" t="inlineStr">
         <is>
-          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
+          <t>Obrázky nahrajte do složky media, která je ve složce klienta vedle této tabulky. Podsložky jsou v pořádku.</t>
         </is>
       </c>
     </row>
@@ -1861,7 +1871,7 @@
       </c>
       <c r="B87" s="2" t="inlineStr">
         <is>
-          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
+          <t>V tabulce pak stačí název souboru: hero.jpg. Když je stejný název ve dvou podsložkách, napište cestu: galerie/hero.jpg.</t>
         </is>
       </c>
     </row>
@@ -1873,7 +1883,7 @@
       </c>
       <c r="B88" s="2" t="inlineStr">
         <is>
-          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+          <t>Web obrázky sám zmenší a převede do rychlých formátů. Nahrávejte je v plné kvalitě, nic neupravujte.</t>
         </is>
       </c>
     </row>
@@ -1885,26 +1895,26 @@
       </c>
       <c r="B89" s="2" t="inlineStr">
         <is>
+          <t>Používejte JPG, PNG nebo WebP. Fotky z iPhonu (HEIC) převeďte, nebo v iPhonu nastavte Fotoaparát → Formáty → Nejkompatibilnější.</t>
+        </is>
+      </c>
+    </row>
+    <row r="90" ht="28" customHeight="1">
+      <c r="A90" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B90" s="2" t="inlineStr">
+        <is>
           <t>Videa dávejte na YouTube nebo Vimeo a do stránky vložte odkaz.</t>
         </is>
       </c>
     </row>
-    <row r="91">
-      <c r="A91" s="3" t="inlineStr">
+    <row r="92">
+      <c r="A92" s="3" t="inlineStr">
         <is>
           <t>Publikování</t>
-        </is>
-      </c>
-    </row>
-    <row r="92" ht="28" customHeight="1">
-      <c r="A92" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B92" s="2" t="inlineStr">
-        <is>
-          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1916,7 +1926,7 @@
       </c>
       <c r="B93" s="2" t="inlineStr">
         <is>
-          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+          <t>Až budete s úpravami hotovi, klikněte v horním menu na Web → Publikovat. Za minutu až dvě je web online.</t>
         </is>
       </c>
     </row>
@@ -1928,26 +1938,26 @@
       </c>
       <c r="B94" s="2" t="inlineStr">
         <is>
+          <t>Výsledek se objeví v listu stav: kdy se publikovalo, jestli vše proběhlo a případná upozornění (třeba chybějící obrázek).</t>
+        </is>
+      </c>
+    </row>
+    <row r="95" ht="28" customHeight="1">
+      <c r="A95" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B95" s="2" t="inlineStr">
+        <is>
           <t>Dokud nekliknete na Publikovat, návštěvníci vidí předchozí verzi. Upravovat tedy můžete v klidu.</t>
         </is>
       </c>
     </row>
-    <row r="96">
-      <c r="A96" s="3" t="inlineStr">
+    <row r="97">
+      <c r="A97" s="3" t="inlineStr">
         <is>
           <t>Pravidla</t>
-        </is>
-      </c>
-    </row>
-    <row r="97" ht="28" customHeight="1">
-      <c r="A97" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B97" s="2" t="inlineStr">
-        <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -1959,7 +1969,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -1971,7 +1981,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
         </is>
       </c>
     </row>
@@ -1983,7 +1993,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
         </is>
       </c>
     </row>
@@ -1995,7 +2005,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
         </is>
       </c>
     </row>
@@ -2007,64 +2017,76 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="103" ht="28" customHeight="1">
+      <c r="A103" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B103" s="2" t="inlineStr">
+        <is>
           <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
         </is>
       </c>
     </row>
-    <row r="104">
-      <c r="A104" s="3" t="inlineStr">
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
         <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="8" t="inlineStr">
+    <row r="106">
+      <c r="A106" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr"/>
-      <c r="C105" s="2" t="inlineStr">
-        <is>
-          <t>Obsah stránky a texty. Tady skládáte.</t>
-        </is>
-      </c>
-    </row>
-    <row r="106">
-      <c r="A106" s="2" t="inlineStr">
-        <is>
-          <t>bílé buňky</t>
         </is>
       </c>
       <c r="B106" s="2" t="inlineStr"/>
       <c r="C106" s="2" t="inlineStr">
         <is>
-          <t>Nastavení a údaje.</t>
+          <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
     <row r="107">
-      <c r="A107" s="9" t="inlineStr">
-        <is>
-          <t>šedé buňky</t>
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>bílé buňky</t>
         </is>
       </c>
       <c r="B107" s="2" t="inlineStr"/>
       <c r="C107" s="2" t="inlineStr">
         <is>
-          <t>Poznámky pro vás. Na webu se neobjeví.</t>
+          <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
     <row r="108">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>roletky</t>
+      <c r="A108" s="9" t="inlineStr">
+        <is>
+          <t>šedé buňky</t>
         </is>
       </c>
       <c r="B108" s="2" t="inlineStr"/>
       <c r="C108" s="2" t="inlineStr">
+        <is>
+          <t>Poznámky pro vás. Na webu se neobjeví.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>roletky</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr"/>
+      <c r="C109" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
@@ -2077,21 +2099,21 @@
     <mergeCell ref="B101:D101"/>
     <mergeCell ref="B88:D88"/>
     <mergeCell ref="B87:D87"/>
+    <mergeCell ref="B103:D103"/>
     <mergeCell ref="B99:D99"/>
     <mergeCell ref="A15:D15"/>
-    <mergeCell ref="A59:D59"/>
-    <mergeCell ref="B92:D92"/>
+    <mergeCell ref="A60:D60"/>
+    <mergeCell ref="B95:D95"/>
     <mergeCell ref="B89:D89"/>
+    <mergeCell ref="A79:D79"/>
     <mergeCell ref="B94:D94"/>
-    <mergeCell ref="B85:D85"/>
-    <mergeCell ref="A78:D78"/>
-    <mergeCell ref="B97:D97"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="B100:D100"/>
-    <mergeCell ref="A56:D56"/>
+    <mergeCell ref="B90:D90"/>
     <mergeCell ref="B102:D102"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="B93:D93"/>
+    <mergeCell ref="A57:D57"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B86:D86"/>
   </mergeCells>
@@ -6455,10 +6477,34 @@
       </c>
     </row>
     <row r="11">
-      <c r="C11" s="15" t="n"/>
+      <c r="A11" s="11" t="inlineStr">
+        <is>
+          <t>address</t>
+        </is>
+      </c>
+      <c r="B11" s="5" t="inlineStr"/>
+      <c r="C11" s="13" t="inlineStr">
+        <is>
+          <t>Adresa pro mapu (mapa:), např. Vinohradská 12, Praha 2. Na webu se zobrazí pod mapou.</t>
+        </is>
+      </c>
     </row>
     <row r="12">
-      <c r="C12" s="15" t="n"/>
+      <c r="A12" s="11" t="inlineStr">
+        <is>
+          <t>map_zoom</t>
+        </is>
+      </c>
+      <c r="B12" s="5" t="inlineStr">
+        <is>
+          <t>15</t>
+        </is>
+      </c>
+      <c r="C12" s="13" t="inlineStr">
+        <is>
+          <t>Přiblížení mapy: 1 = celý svět, 15 = ulice, 18 = dům.</t>
+        </is>
+      </c>
     </row>
     <row r="13">
       <c r="C13" s="15" t="n"/>

</xml_diff>

<commit_message>
Více jazyků: překlad ve sloupcích _en, přepínač, /en/ adresy
site › languages (cs, en) zapne další jazyky; první je hlavní. Překlad se
píše do sloupců s koncovkou jazyka (title_en, content_en, text_en …),
id_en dává anglickou adresu (/en/why-us/). Chybějící překlad se nahradí
původním textem a hlásí se v listu stav.

Na webu: přepínač CS · EN u záložek, který jde vždy na tutéž stránku,
hreflang pro vyhledávače, společná mapa webu. Prohlížeč nastavený na jiný
jazyk webu se napoprvé přesměruje, volba v přepínači se pamatuje. Starší
nastavení site › language dál funguje.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fseswgzcM5xGxappQkPY2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D109"/>
+  <dimension ref="A1:D120"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1957,7 +1957,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Pravidla</t>
+          <t>Více jazyků</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
+          <t>V listu site napište do languages všechny jazyky, první je hlavní: cs, en. Hlavní jazyk je na adrese webu, další pod /en/.</t>
         </is>
       </c>
     </row>
@@ -1981,7 +1981,7 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+          <t>Překlad píšete do sloupců s koncovkou jazyka vedle původních: tab_label_en, title_en, content_en, description_en v pages, content_en v texts, title_en a text_en v items, alt_en v media, html_en v embeds.</t>
         </is>
       </c>
     </row>
@@ -1993,7 +1993,7 @@
       </c>
       <c r="B100" s="2" t="inlineStr">
         <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+          <t>id_en v pages je adresa stránky v angličtině, např. why-us → /en/why-us/. Prázdné = stejné id jako v češtině.</t>
         </is>
       </c>
     </row>
@@ -2005,7 +2005,7 @@
       </c>
       <c r="B101" s="2" t="inlineStr">
         <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>Odkazy v překladu můžete psát s českým i anglickým id (/proc-s-nami/ i /why-us/), vždy povedou na anglickou verzi stránky.</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2017,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>visible_en: no skryje stránku nebo položku jen v angličtině.</t>
         </is>
       </c>
     </row>
@@ -2029,93 +2029,217 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
+          <t>Obrázky, barvy, pořadí a nastavení vzhledu jsou společné. V content_en stačí napsat stejné obrázky a galerie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="104" ht="28" customHeight="1">
+      <c r="A104" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B104" s="2" t="inlineStr">
+        <is>
+          <t>Chybí-li překlad, zobrazí se původní text a v listu stav se objeví upozornění.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105" ht="28" customHeight="1">
+      <c r="A105" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B105" s="2" t="inlineStr">
+        <is>
+          <t>Návštěvník přepíná jazyk u záložek. Má-li prohlížeč nastavený jiný jazyk webu, otevře se mu napoprvé rovnou ten. Jeho volba se pamatuje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="106" ht="28" customHeight="1">
+      <c r="A106" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B106" s="2" t="inlineStr">
+        <is>
+          <t>V site můžete přeložit i site_name_en, description_en a footer_en.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108">
+      <c r="A108" s="3" t="inlineStr">
+        <is>
+          <t>Pravidla</t>
+        </is>
+      </c>
+    </row>
+    <row r="109" ht="28" customHeight="1">
+      <c r="A109" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B109" s="2" t="inlineStr">
+        <is>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
+        </is>
+      </c>
+    </row>
+    <row r="110" ht="28" customHeight="1">
+      <c r="A110" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B110" s="2" t="inlineStr">
+        <is>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="28" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="28" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="113" ht="28" customHeight="1">
+      <c r="A113" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B113" s="2" t="inlineStr">
+        <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="114" ht="28" customHeight="1">
+      <c r="A114" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B114" s="2" t="inlineStr">
+        <is>
           <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
         </is>
       </c>
     </row>
-    <row r="105">
-      <c r="A105" s="3" t="inlineStr">
+    <row r="116">
+      <c r="A116" s="3" t="inlineStr">
         <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="106">
-      <c r="A106" s="8" t="inlineStr">
+    <row r="117">
+      <c r="A117" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
         </is>
       </c>
-      <c r="B106" s="2" t="inlineStr"/>
-      <c r="C106" s="2" t="inlineStr">
+      <c r="B117" s="2" t="inlineStr"/>
+      <c r="C117" s="2" t="inlineStr">
         <is>
           <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
-    <row r="107">
-      <c r="A107" s="2" t="inlineStr">
+    <row r="118">
+      <c r="A118" s="2" t="inlineStr">
         <is>
           <t>bílé buňky</t>
         </is>
       </c>
-      <c r="B107" s="2" t="inlineStr"/>
-      <c r="C107" s="2" t="inlineStr">
+      <c r="B118" s="2" t="inlineStr"/>
+      <c r="C118" s="2" t="inlineStr">
         <is>
           <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
-    <row r="108">
-      <c r="A108" s="9" t="inlineStr">
+    <row r="119">
+      <c r="A119" s="9" t="inlineStr">
         <is>
           <t>šedé buňky</t>
         </is>
       </c>
-      <c r="B108" s="2" t="inlineStr"/>
-      <c r="C108" s="2" t="inlineStr">
+      <c r="B119" s="2" t="inlineStr"/>
+      <c r="C119" s="2" t="inlineStr">
         <is>
           <t>Poznámky pro vás. Na webu se neobjeví.</t>
         </is>
       </c>
     </row>
-    <row r="109">
-      <c r="A109" s="2" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="2" t="inlineStr">
         <is>
           <t>roletky</t>
         </is>
       </c>
-      <c r="B109" s="2" t="inlineStr"/>
-      <c r="C109" s="2" t="inlineStr">
+      <c r="B120" s="2" t="inlineStr"/>
+      <c r="C120" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="22">
+  <mergeCells count="31">
     <mergeCell ref="B98:D98"/>
     <mergeCell ref="A35:D35"/>
     <mergeCell ref="B101:D101"/>
     <mergeCell ref="B88:D88"/>
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="B103:D103"/>
+    <mergeCell ref="B112:D112"/>
     <mergeCell ref="B99:D99"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="B95:D95"/>
     <mergeCell ref="B89:D89"/>
+    <mergeCell ref="B104:D104"/>
     <mergeCell ref="A79:D79"/>
+    <mergeCell ref="B114:D114"/>
     <mergeCell ref="B94:D94"/>
+    <mergeCell ref="B110:D110"/>
     <mergeCell ref="A25:D25"/>
     <mergeCell ref="B100:D100"/>
+    <mergeCell ref="B106:D106"/>
+    <mergeCell ref="B113:D113"/>
+    <mergeCell ref="B109:D109"/>
     <mergeCell ref="B90:D90"/>
     <mergeCell ref="B102:D102"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="B93:D93"/>
     <mergeCell ref="A57:D57"/>
+    <mergeCell ref="B105:D105"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B86:D86"/>
+    <mergeCell ref="B111:D111"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -6347,7 +6471,7 @@
     <row r="3">
       <c r="A3" s="11" t="inlineStr">
         <is>
-          <t>language</t>
+          <t>languages</t>
         </is>
       </c>
       <c r="B3" s="5" t="inlineStr">
@@ -6357,7 +6481,7 @@
       </c>
       <c r="C3" s="13" t="inlineStr">
         <is>
-          <t>Hlavní jazyk webu: cs nebo en. Ovlivní dělení slov a formát dat.</t>
+          <t>Jazyky webu, první je hlavní: cs, nebo cs, en. Další jazyk píšete do sloupců s koncovkou _en (viz Návod › Více jazyků).</t>
         </is>
       </c>
     </row>

</xml_diff>

<commit_message>
Široký obsah: náhled na stránce, celý ve vrstvě nad knihou
Na počítači web po zobrazení stránky změří vložené prvky. Co se nevejde
na šířku stránky (široká tabulka, widget), zůstane jako náhled, který
doprava plynule mizí, s tlačítkem Zobrazit celé. Kliknutí otevře obsah
na skleněném listu nad ztmavenou knihou v barvě stránky; zavírá se
křížkem, Esc nebo kliknutím mimo. Obsah se přesouvá, ne kopíruje, takže
formuláře a widgety si drží stav. Na mobilu beze změny.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fseswgzcM5xGxappQkPY2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D120"/>
+  <dimension ref="A1:D124"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1957,7 +1957,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Více jazyků</t>
+          <t>Široký obsah</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>V listu site napište do languages všechny jazyky, první je hlavní: cs, en. Hlavní jazyk je na adrese webu, další pod /en/.</t>
+          <t>Když se vložený prvek (embed) nevejde na šířku stránky, třeba široká tabulka, zobrazí se na počítači jako náhled s tlačítkem Zobrazit celé. Po kliknutí se otevře celý ve vrstvě nad knihou.</t>
         </is>
       </c>
     </row>
@@ -1981,31 +1981,14 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Překlad píšete do sloupců s koncovkou jazyka vedle původních: tab_label_en, title_en, content_en, description_en v pages, content_en v texts, title_en a text_en v items, alt_en v media, html_en v embeds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="100" ht="28" customHeight="1">
-      <c r="A100" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B100" s="2" t="inlineStr">
-        <is>
-          <t>id_en v pages je adresa stránky v angličtině, např. why-us → /en/why-us/. Prázdné = stejné id jako v češtině.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101" ht="28" customHeight="1">
-      <c r="A101" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B101" s="2" t="inlineStr">
-        <is>
-          <t>Odkazy v překladu můžete psát s českým i anglickým id (/proc-s-nami/ i /why-us/), vždy povedou na anglickou verzi stránky.</t>
+          <t>Nic se nenastavuje, web to pozná sám. Na mobilu se široký obsah posouvá prstem do strany.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101">
+      <c r="A101" s="3" t="inlineStr">
+        <is>
+          <t>Více jazyků</t>
         </is>
       </c>
     </row>
@@ -2017,7 +2000,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>visible_en: no skryje stránku nebo položku jen v angličtině.</t>
+          <t>V listu site napište do languages všechny jazyky, první je hlavní: cs, en. Hlavní jazyk je na adrese webu, další pod /en/.</t>
         </is>
       </c>
     </row>
@@ -2029,7 +2012,7 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Obrázky, barvy, pořadí a nastavení vzhledu jsou společné. V content_en stačí napsat stejné obrázky a galerie.</t>
+          <t>Překlad píšete do sloupců s koncovkou jazyka vedle původních: tab_label_en, title_en, content_en, description_en v pages, content_en v texts, title_en a text_en v items, alt_en v media, html_en v embeds.</t>
         </is>
       </c>
     </row>
@@ -2041,7 +2024,7 @@
       </c>
       <c r="B104" s="2" t="inlineStr">
         <is>
-          <t>Chybí-li překlad, zobrazí se původní text a v listu stav se objeví upozornění.</t>
+          <t>id_en v pages je adresa stránky v angličtině, např. why-us → /en/why-us/. Prázdné = stejné id jako v češtině.</t>
         </is>
       </c>
     </row>
@@ -2053,7 +2036,7 @@
       </c>
       <c r="B105" s="2" t="inlineStr">
         <is>
-          <t>Jazyk se dá přepnout odkazem v patičce (English / Česky). Má-li prohlížeč nastavený jiný jazyk webu, otevře se mu napoprvé rovnou ten. Jeho volba se pamatuje.</t>
+          <t>Odkazy v překladu můžete psát s českým i anglickým id (/proc-s-nami/ i /why-us/), vždy povedou na anglickou verzi stránky.</t>
         </is>
       </c>
     </row>
@@ -2065,14 +2048,31 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>V site můžete přeložit i site_name_en, description_en a footer_en.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108">
-      <c r="A108" s="3" t="inlineStr">
-        <is>
-          <t>Pravidla</t>
+          <t>visible_en: no skryje stránku nebo položku jen v angličtině.</t>
+        </is>
+      </c>
+    </row>
+    <row r="107" ht="28" customHeight="1">
+      <c r="A107" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B107" s="2" t="inlineStr">
+        <is>
+          <t>Obrázky, barvy, pořadí a nastavení vzhledu jsou společné. V content_en stačí napsat stejné obrázky a galerie.</t>
+        </is>
+      </c>
+    </row>
+    <row r="108" ht="28" customHeight="1">
+      <c r="A108" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B108" s="2" t="inlineStr">
+        <is>
+          <t>Chybí-li překlad, zobrazí se původní text a v listu stav se objeví upozornění.</t>
         </is>
       </c>
     </row>
@@ -2084,7 +2084,7 @@
       </c>
       <c r="B109" s="2" t="inlineStr">
         <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
+          <t>Jazyk se dá přepnout odkazem v patičce (English / Česky). Má-li prohlížeč nastavený jiný jazyk webu, otevře se mu napoprvé rovnou ten. Jeho volba se pamatuje.</t>
         </is>
       </c>
     </row>
@@ -2096,31 +2096,14 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
-        </is>
-      </c>
-    </row>
-    <row r="111" ht="28" customHeight="1">
-      <c r="A111" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B111" s="2" t="inlineStr">
-        <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
-        </is>
-      </c>
-    </row>
-    <row r="112" ht="28" customHeight="1">
-      <c r="A112" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B112" s="2" t="inlineStr">
-        <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>V site můžete přeložit i site_name_en, description_en a footer_en.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112">
+      <c r="A112" s="3" t="inlineStr">
+        <is>
+          <t>Pravidla</t>
         </is>
       </c>
     </row>
@@ -2132,7 +2115,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
         </is>
       </c>
     </row>
@@ -2144,79 +2127,130 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="115" ht="28" customHeight="1">
+      <c r="A115" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B115" s="2" t="inlineStr">
+        <is>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="116" ht="28" customHeight="1">
+      <c r="A116" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B116" s="2" t="inlineStr">
+        <is>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="117" ht="28" customHeight="1">
+      <c r="A117" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B117" s="2" t="inlineStr">
+        <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="118" ht="28" customHeight="1">
+      <c r="A118" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B118" s="2" t="inlineStr">
+        <is>
           <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
         </is>
       </c>
     </row>
-    <row r="116">
-      <c r="A116" s="3" t="inlineStr">
+    <row r="120">
+      <c r="A120" s="3" t="inlineStr">
         <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="117">
-      <c r="A117" s="8" t="inlineStr">
+    <row r="121">
+      <c r="A121" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
         </is>
       </c>
-      <c r="B117" s="2" t="inlineStr"/>
-      <c r="C117" s="2" t="inlineStr">
+      <c r="B121" s="2" t="inlineStr"/>
+      <c r="C121" s="2" t="inlineStr">
         <is>
           <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
-    <row r="118">
-      <c r="A118" s="2" t="inlineStr">
+    <row r="122">
+      <c r="A122" s="2" t="inlineStr">
         <is>
           <t>bílé buňky</t>
         </is>
       </c>
-      <c r="B118" s="2" t="inlineStr"/>
-      <c r="C118" s="2" t="inlineStr">
+      <c r="B122" s="2" t="inlineStr"/>
+      <c r="C122" s="2" t="inlineStr">
         <is>
           <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
-    <row r="119">
-      <c r="A119" s="9" t="inlineStr">
+    <row r="123">
+      <c r="A123" s="9" t="inlineStr">
         <is>
           <t>šedé buňky</t>
         </is>
       </c>
-      <c r="B119" s="2" t="inlineStr"/>
-      <c r="C119" s="2" t="inlineStr">
+      <c r="B123" s="2" t="inlineStr"/>
+      <c r="C123" s="2" t="inlineStr">
         <is>
           <t>Poznámky pro vás. Na webu se neobjeví.</t>
         </is>
       </c>
     </row>
-    <row r="120">
-      <c r="A120" s="2" t="inlineStr">
+    <row r="124">
+      <c r="A124" s="2" t="inlineStr">
         <is>
           <t>roletky</t>
         </is>
       </c>
-      <c r="B120" s="2" t="inlineStr"/>
-      <c r="C120" s="2" t="inlineStr">
+      <c r="B124" s="2" t="inlineStr"/>
+      <c r="C124" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="31">
+  <mergeCells count="33">
     <mergeCell ref="B98:D98"/>
+    <mergeCell ref="B107:D107"/>
     <mergeCell ref="A35:D35"/>
-    <mergeCell ref="B101:D101"/>
+    <mergeCell ref="B117:D117"/>
     <mergeCell ref="B88:D88"/>
+    <mergeCell ref="B116:D116"/>
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="B103:D103"/>
-    <mergeCell ref="B112:D112"/>
+    <mergeCell ref="B108:D108"/>
     <mergeCell ref="B99:D99"/>
+    <mergeCell ref="B118:D118"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="B95:D95"/>
@@ -2227,19 +2261,18 @@
     <mergeCell ref="B94:D94"/>
     <mergeCell ref="B110:D110"/>
     <mergeCell ref="A25:D25"/>
-    <mergeCell ref="B100:D100"/>
     <mergeCell ref="B106:D106"/>
     <mergeCell ref="B113:D113"/>
     <mergeCell ref="B109:D109"/>
     <mergeCell ref="B90:D90"/>
     <mergeCell ref="B102:D102"/>
+    <mergeCell ref="B115:D115"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="B93:D93"/>
     <mergeCell ref="A57:D57"/>
     <mergeCell ref="B105:D105"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B86:D86"/>
-    <mergeCell ref="B111:D111"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>

</xml_diff>

<commit_message>
Podstránky: sloupec parent_page, menu na listu hlavní stránky
Řádek v pages s parent_page je podstránka své hlavní stránky. Nemá
záložku; zobrazí se na listu hlavní stránky za jejím obsahem, za menu
podstránek. Menu se při čtení drží u horní hrany listu (na mobilu pod
záložkami), zvýrazňuje čtenou podstránku a první položka vede nahoru.

Každá podstránka má vlastní adresu (/hlavni/podstranka/), titulek,
popis, hreflang a místo v mapě webu; adresa se při čtení tiše mění,
Zpět funguje. Odkaz /podstranka/ odkudkoli otočí list a sjede na místo.
Po dojetí se cíl přeměří a doladí, pokud se obsah nad ním mezitím
změnil. Jen jedna úroveň; chybné parent_page hlásí list stav.

Co-Authored-By: Claude Opus 5.5 <noreply@anthropic.com>
Claude-Session: https://claude.ai/code/session_012fseswgzcM5xGxappQkPY2
</commit_message>
<xml_diff>
--- a/templates/klient-sablona.xlsx
+++ b/templates/klient-sablona.xlsx
@@ -513,7 +513,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:D124"/>
+  <dimension ref="A1:D132"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="22" customWidth="1" min="1" max="1"/>
@@ -1957,7 +1957,7 @@
     <row r="97">
       <c r="A97" s="3" t="inlineStr">
         <is>
-          <t>Široký obsah</t>
+          <t>Podstránky</t>
         </is>
       </c>
     </row>
@@ -1969,7 +1969,7 @@
       </c>
       <c r="B98" s="2" t="inlineStr">
         <is>
-          <t>Když se vložený prvek (embed) nevejde na šířku stránky, třeba široká tabulka, zobrazí se na počítači jako náhled s tlačítkem Zobrazit celé. Po kliknutí se otevře celý ve vrstvě nad knihou.</t>
+          <t>Podstránka je řádek v pages, který má ve sloupci parent_page id hlavní stránky. Prázdné parent_page = hlavní stránka se záložkou.</t>
         </is>
       </c>
     </row>
@@ -1981,14 +1981,31 @@
       </c>
       <c r="B99" s="2" t="inlineStr">
         <is>
-          <t>Nic se nenastavuje, web to pozná sám. Na mobilu se široký obsah posouvá prstem do strany.</t>
-        </is>
-      </c>
-    </row>
-    <row r="101">
-      <c r="A101" s="3" t="inlineStr">
-        <is>
-          <t>Více jazyků</t>
+          <t>Podstránky nemají vlastní záložku. Zobrazí se na listu své hlavní stránky: nejdřív obsah hlavní stránky, pak menu, pak podstránky za sebou.</t>
+        </is>
+      </c>
+    </row>
+    <row r="100" ht="28" customHeight="1">
+      <c r="A100" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B100" s="2" t="inlineStr">
+        <is>
+          <t>Menu se při čtení drží nahoře na listu a ukazuje, kde čtenář je. První položka (tab_label hlavní stránky) vede zpět nahoru.</t>
+        </is>
+      </c>
+    </row>
+    <row r="101" ht="28" customHeight="1">
+      <c r="A101" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B101" s="2" t="inlineStr">
+        <is>
+          <t>order u podstránky určuje pořadí v rámci její hlavní stránky. tab_label je krátký název v menu, title nadpis podstránky, hue se nepoužije.</t>
         </is>
       </c>
     </row>
@@ -2000,7 +2017,7 @@
       </c>
       <c r="B102" s="2" t="inlineStr">
         <is>
-          <t>V listu site napište do languages všechny jazyky, první je hlavní: cs, en. Hlavní jazyk je na adrese webu, další pod /en/.</t>
+          <t>Každá podstránka má vlastní adresu, např. /jak-to-probiha/konzultace/. V odkazech stačí psát /konzultace/.</t>
         </is>
       </c>
     </row>
@@ -2012,31 +2029,14 @@
       </c>
       <c r="B103" s="2" t="inlineStr">
         <is>
-          <t>Překlad píšete do sloupců s koncovkou jazyka vedle původních: tab_label_en, title_en, content_en, description_en v pages, content_en v texts, title_en a text_en v items, alt_en v media, html_en v embeds.</t>
-        </is>
-      </c>
-    </row>
-    <row r="104" ht="28" customHeight="1">
-      <c r="A104" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B104" s="2" t="inlineStr">
-        <is>
-          <t>id_en v pages je adresa stránky v angličtině, např. why-us → /en/why-us/. Prázdné = stejné id jako v češtině.</t>
-        </is>
-      </c>
-    </row>
-    <row r="105" ht="28" customHeight="1">
-      <c r="A105" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B105" s="2" t="inlineStr">
-        <is>
-          <t>Odkazy v překladu můžete psát s českým i anglickým id (/proc-s-nami/ i /why-us/), vždy povedou na anglickou verzi stránky.</t>
+          <t>Podstránky jsou jen o jednu úroveň. Jako home_page nastavte vždy hlavní stránku.</t>
+        </is>
+      </c>
+    </row>
+    <row r="105">
+      <c r="A105" s="3" t="inlineStr">
+        <is>
+          <t>Široký obsah</t>
         </is>
       </c>
     </row>
@@ -2048,7 +2048,7 @@
       </c>
       <c r="B106" s="2" t="inlineStr">
         <is>
-          <t>visible_en: no skryje stránku nebo položku jen v angličtině.</t>
+          <t>Když se vložený prvek (embed) nevejde na šířku stránky, třeba široká tabulka, zobrazí se na počítači jako náhled s tlačítkem Zobrazit celé. Po kliknutí se otevře celý ve vrstvě nad knihou.</t>
         </is>
       </c>
     </row>
@@ -2060,31 +2060,14 @@
       </c>
       <c r="B107" s="2" t="inlineStr">
         <is>
-          <t>Obrázky, barvy, pořadí a nastavení vzhledu jsou společné. V content_en stačí napsat stejné obrázky a galerie.</t>
-        </is>
-      </c>
-    </row>
-    <row r="108" ht="28" customHeight="1">
-      <c r="A108" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B108" s="2" t="inlineStr">
-        <is>
-          <t>Chybí-li překlad, zobrazí se původní text a v listu stav se objeví upozornění.</t>
-        </is>
-      </c>
-    </row>
-    <row r="109" ht="28" customHeight="1">
-      <c r="A109" s="2" t="inlineStr">
-        <is>
-          <t>•</t>
-        </is>
-      </c>
-      <c r="B109" s="2" t="inlineStr">
-        <is>
-          <t>Jazyk se dá přepnout odkazem v patičce (English / Česky). Má-li prohlížeč nastavený jiný jazyk webu, otevře se mu napoprvé rovnou ten. Jeho volba se pamatuje.</t>
+          <t>Nic se nenastavuje, web to pozná sám. Na mobilu se široký obsah posouvá prstem do strany.</t>
+        </is>
+      </c>
+    </row>
+    <row r="109">
+      <c r="A109" s="3" t="inlineStr">
+        <is>
+          <t>Více jazyků</t>
         </is>
       </c>
     </row>
@@ -2096,14 +2079,31 @@
       </c>
       <c r="B110" s="2" t="inlineStr">
         <is>
-          <t>V site můžete přeložit i site_name_en, description_en a footer_en.</t>
-        </is>
-      </c>
-    </row>
-    <row r="112">
-      <c r="A112" s="3" t="inlineStr">
-        <is>
-          <t>Pravidla</t>
+          <t>V listu site napište do languages všechny jazyky, první je hlavní: cs, en. Hlavní jazyk je na adrese webu, další pod /en/.</t>
+        </is>
+      </c>
+    </row>
+    <row r="111" ht="28" customHeight="1">
+      <c r="A111" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B111" s="2" t="inlineStr">
+        <is>
+          <t>Překlad píšete do sloupců s koncovkou jazyka vedle původních: tab_label_en, title_en, content_en, description_en v pages, content_en v texts, title_en a text_en v items, alt_en v media, html_en v embeds.</t>
+        </is>
+      </c>
+    </row>
+    <row r="112" ht="28" customHeight="1">
+      <c r="A112" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B112" s="2" t="inlineStr">
+        <is>
+          <t>id_en v pages je adresa stránky v angličtině, např. why-us → /en/why-us/. Prázdné = stejné id jako v češtině.</t>
         </is>
       </c>
     </row>
@@ -2115,7 +2115,7 @@
       </c>
       <c r="B113" s="2" t="inlineStr">
         <is>
-          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
+          <t>Odkazy v překladu můžete psát s českým i anglickým id (/proc-s-nami/ i /why-us/), vždy povedou na anglickou verzi stránky.</t>
         </is>
       </c>
     </row>
@@ -2127,7 +2127,7 @@
       </c>
       <c r="B114" s="2" t="inlineStr">
         <is>
-          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+          <t>visible_en: no skryje stránku nebo položku jen v angličtině.</t>
         </is>
       </c>
     </row>
@@ -2139,7 +2139,7 @@
       </c>
       <c r="B115" s="2" t="inlineStr">
         <is>
-          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+          <t>Obrázky, barvy, pořadí a nastavení vzhledu jsou společné. V content_en stačí napsat stejné obrázky a galerie.</t>
         </is>
       </c>
     </row>
@@ -2151,7 +2151,7 @@
       </c>
       <c r="B116" s="2" t="inlineStr">
         <is>
-          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+          <t>Chybí-li překlad, zobrazí se původní text a v listu stav se objeví upozornění.</t>
         </is>
       </c>
     </row>
@@ -2163,7 +2163,7 @@
       </c>
       <c r="B117" s="2" t="inlineStr">
         <is>
-          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+          <t>Jazyk se dá přepnout odkazem v patičce (English / Česky). Má-li prohlížeč nastavený jiný jazyk webu, otevře se mu napoprvé rovnou ten. Jeho volba se pamatuje.</t>
         </is>
       </c>
     </row>
@@ -2175,104 +2175,189 @@
       </c>
       <c r="B118" s="2" t="inlineStr">
         <is>
-          <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
+          <t>V site můžete přeložit i site_name_en, description_en a footer_en.</t>
         </is>
       </c>
     </row>
     <row r="120">
       <c r="A120" s="3" t="inlineStr">
         <is>
+          <t>Pravidla</t>
+        </is>
+      </c>
+    </row>
+    <row r="121" ht="28" customHeight="1">
+      <c r="A121" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B121" s="2" t="inlineStr">
+        <is>
+          <t>id: malá písmena, bez mezer a diakritiky, slova spojená pomlčkou (t-intro, img-hero).</t>
+        </is>
+      </c>
+    </row>
+    <row r="122" ht="28" customHeight="1">
+      <c r="A122" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B122" s="2" t="inlineStr">
+        <is>
+          <t>order: počítejte po desítkách (10, 20, 30). Když později něco vložíte mezi, dáte 15 a nic se nepřečísluje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="123" ht="28" customHeight="1">
+      <c r="A123" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B123" s="2" t="inlineStr">
+        <is>
+          <t>visible: no skryje stránku nebo položku, aniž byste ji mazali.</t>
+        </is>
+      </c>
+    </row>
+    <row r="124" ht="28" customHeight="1">
+      <c r="A124" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B124" s="2" t="inlineStr">
+        <is>
+          <t>Klíčové slovo s dvojtečkou vždy začíná nový kus. Nepište proto „poznámka:“ uprostřed běžné věty.</t>
+        </is>
+      </c>
+    </row>
+    <row r="125" ht="28" customHeight="1">
+      <c r="A125" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B125" s="2" t="inlineStr">
+        <is>
+          <t>Názvy sloupců (tmavé záhlaví) neměňte, web je podle nich čte.</t>
+        </is>
+      </c>
+    </row>
+    <row r="126" ht="28" customHeight="1">
+      <c r="A126" s="2" t="inlineStr">
+        <is>
+          <t>•</t>
+        </is>
+      </c>
+      <c r="B126" s="2" t="inlineStr">
+        <is>
+          <t>Pod patičkou každé stránky je drobný odkaz platform by filipmracek.com. Ten je součástí platformy, v tabulce se nenastavuje.</t>
+        </is>
+      </c>
+    </row>
+    <row r="128">
+      <c r="A128" s="3" t="inlineStr">
+        <is>
           <t>Barvy v tabulce</t>
         </is>
       </c>
     </row>
-    <row r="121">
-      <c r="A121" s="8" t="inlineStr">
+    <row r="129">
+      <c r="A129" s="8" t="inlineStr">
         <is>
           <t>žluté buňky</t>
         </is>
       </c>
-      <c r="B121" s="2" t="inlineStr"/>
-      <c r="C121" s="2" t="inlineStr">
+      <c r="B129" s="2" t="inlineStr"/>
+      <c r="C129" s="2" t="inlineStr">
         <is>
           <t>Obsah stránky a texty. Tady skládáte.</t>
         </is>
       </c>
     </row>
-    <row r="122">
-      <c r="A122" s="2" t="inlineStr">
+    <row r="130">
+      <c r="A130" s="2" t="inlineStr">
         <is>
           <t>bílé buňky</t>
         </is>
       </c>
-      <c r="B122" s="2" t="inlineStr"/>
-      <c r="C122" s="2" t="inlineStr">
+      <c r="B130" s="2" t="inlineStr"/>
+      <c r="C130" s="2" t="inlineStr">
         <is>
           <t>Nastavení a údaje.</t>
         </is>
       </c>
     </row>
-    <row r="123">
-      <c r="A123" s="9" t="inlineStr">
+    <row r="131">
+      <c r="A131" s="9" t="inlineStr">
         <is>
           <t>šedé buňky</t>
         </is>
       </c>
-      <c r="B123" s="2" t="inlineStr"/>
-      <c r="C123" s="2" t="inlineStr">
+      <c r="B131" s="2" t="inlineStr"/>
+      <c r="C131" s="2" t="inlineStr">
         <is>
           <t>Poznámky pro vás. Na webu se neobjeví.</t>
         </is>
       </c>
     </row>
-    <row r="124">
-      <c r="A124" s="2" t="inlineStr">
+    <row r="132">
+      <c r="A132" s="2" t="inlineStr">
         <is>
           <t>roletky</t>
         </is>
       </c>
-      <c r="B124" s="2" t="inlineStr"/>
-      <c r="C124" s="2" t="inlineStr">
+      <c r="B132" s="2" t="inlineStr"/>
+      <c r="C132" s="2" t="inlineStr">
         <is>
           <t>Sloupce jako visible, kind a focus berou jen nabízené hodnoty.</t>
         </is>
       </c>
     </row>
   </sheetData>
-  <mergeCells count="33">
+  <mergeCells count="39">
     <mergeCell ref="B98:D98"/>
     <mergeCell ref="B107:D107"/>
     <mergeCell ref="A35:D35"/>
+    <mergeCell ref="B101:D101"/>
     <mergeCell ref="B117:D117"/>
     <mergeCell ref="B88:D88"/>
     <mergeCell ref="B116:D116"/>
     <mergeCell ref="B87:D87"/>
     <mergeCell ref="B103:D103"/>
-    <mergeCell ref="B108:D108"/>
+    <mergeCell ref="B112:D112"/>
     <mergeCell ref="B99:D99"/>
     <mergeCell ref="B118:D118"/>
     <mergeCell ref="A15:D15"/>
     <mergeCell ref="A60:D60"/>
     <mergeCell ref="B95:D95"/>
     <mergeCell ref="B89:D89"/>
-    <mergeCell ref="B104:D104"/>
+    <mergeCell ref="B124:D124"/>
     <mergeCell ref="A79:D79"/>
     <mergeCell ref="B114:D114"/>
     <mergeCell ref="B94:D94"/>
     <mergeCell ref="B110:D110"/>
+    <mergeCell ref="B123:D123"/>
     <mergeCell ref="A25:D25"/>
+    <mergeCell ref="B126:D126"/>
+    <mergeCell ref="B100:D100"/>
     <mergeCell ref="B106:D106"/>
     <mergeCell ref="B113:D113"/>
-    <mergeCell ref="B109:D109"/>
+    <mergeCell ref="B125:D125"/>
     <mergeCell ref="B90:D90"/>
+    <mergeCell ref="B121:D121"/>
+    <mergeCell ref="B122:D122"/>
     <mergeCell ref="B102:D102"/>
     <mergeCell ref="B115:D115"/>
     <mergeCell ref="A26:D26"/>
     <mergeCell ref="B93:D93"/>
     <mergeCell ref="A57:D57"/>
-    <mergeCell ref="B105:D105"/>
     <mergeCell ref="A2:D2"/>
     <mergeCell ref="B86:D86"/>
+    <mergeCell ref="B111:D111"/>
   </mergeCells>
   <pageMargins left="0.75" right="0.75" top="1" bottom="1" header="0.5" footer="0.5"/>
 </worksheet>
@@ -2285,7 +2370,7 @@
     <outlinePr summaryBelow="1" summaryRight="1"/>
     <pageSetUpPr/>
   </sheetPr>
-  <dimension ref="A1:J199"/>
+  <dimension ref="A1:K199"/>
   <sheetFormatPr baseColWidth="8" defaultRowHeight="15"/>
   <cols>
     <col width="12" customWidth="1" min="1" max="1"/>
@@ -2298,6 +2383,7 @@
     <col width="36" customWidth="1" min="8" max="8"/>
     <col width="13" customWidth="1" min="9" max="9"/>
     <col width="30" customWidth="1" min="10" max="10"/>
+    <col width="14" customWidth="1" min="11" max="11"/>
   </cols>
   <sheetData>
     <row r="1" ht="24" customHeight="1">
@@ -2349,6 +2435,11 @@
       <c r="J1" s="10" t="inlineStr">
         <is>
           <t>notes</t>
+        </is>
+      </c>
+      <c r="K1" s="10" t="inlineStr">
+        <is>
+          <t>parent_page</t>
         </is>
       </c>
     </row>

</xml_diff>